<commit_message>
Oct 11, 2026, 12:09 AM
</commit_message>
<xml_diff>
--- a/Bundesliga 26-27.xlsx
+++ b/Bundesliga 26-27.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kuba\Desktop\analityczka\26-27\Bundesliga 26-27\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kuba\Desktop\analityczka\26-27\Ekstraklasa 26-27\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{15110F92-71C5-43ED-9D4C-61F94B869F84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3843870E-5701-4DD8-8438-1571AF6FAF51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{723BE2C8-720D-41E0-A496-B3B96A8488E1}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="483" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="560" uniqueCount="129">
   <si>
     <t>date</t>
   </si>
@@ -417,6 +417,15 @@
   </si>
   <si>
     <t>Sun 20 September, 19:30</t>
+  </si>
+  <si>
+    <t>Fri 9 October, 20:30</t>
+  </si>
+  <si>
+    <t>Sat 10 October, 15:30</t>
+  </si>
+  <si>
+    <t>Sat 10 October, 18:30</t>
   </si>
 </sst>
 </file>
@@ -480,7 +489,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
@@ -496,6 +505,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -831,7 +843,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9ED51FE2-0441-4690-9385-28E7CF18BF79}">
-  <dimension ref="B1:CJ37"/>
+  <dimension ref="B1:CJ44"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="17.7109375" customWidth="1"/>
@@ -1152,7 +1164,7 @@
         <v>59</v>
       </c>
       <c r="H2">
-        <f t="shared" ref="H2:H37" si="0">100-G2</f>
+        <f t="shared" ref="H2:H44" si="0">100-G2</f>
         <v>41</v>
       </c>
       <c r="I2">
@@ -10633,6 +10645,1854 @@
         <v>0</v>
       </c>
       <c r="CJ37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="2:88" x14ac:dyDescent="0.25">
+      <c r="B38" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="D38" t="s">
+        <v>107</v>
+      </c>
+      <c r="E38">
+        <v>2</v>
+      </c>
+      <c r="F38">
+        <v>2</v>
+      </c>
+      <c r="G38">
+        <v>72</v>
+      </c>
+      <c r="H38">
+        <f t="shared" si="0"/>
+        <v>28</v>
+      </c>
+      <c r="I38">
+        <v>2.31</v>
+      </c>
+      <c r="J38">
+        <v>1.31</v>
+      </c>
+      <c r="K38">
+        <v>21</v>
+      </c>
+      <c r="L38">
+        <v>11</v>
+      </c>
+      <c r="M38">
+        <v>9</v>
+      </c>
+      <c r="N38">
+        <v>4</v>
+      </c>
+      <c r="O38">
+        <v>4</v>
+      </c>
+      <c r="P38">
+        <v>2</v>
+      </c>
+      <c r="Q38">
+        <v>2</v>
+      </c>
+      <c r="R38">
+        <v>1</v>
+      </c>
+      <c r="S38">
+        <v>671</v>
+      </c>
+      <c r="T38">
+        <v>216</v>
+      </c>
+      <c r="U38">
+        <v>10</v>
+      </c>
+      <c r="V38">
+        <v>10</v>
+      </c>
+      <c r="W38">
+        <v>9</v>
+      </c>
+      <c r="X38">
+        <v>3</v>
+      </c>
+      <c r="Y38" t="s">
+        <v>90</v>
+      </c>
+      <c r="Z38" t="s">
+        <v>90</v>
+      </c>
+      <c r="AA38">
+        <v>9</v>
+      </c>
+      <c r="AB38">
+        <v>3</v>
+      </c>
+      <c r="AC38">
+        <v>3</v>
+      </c>
+      <c r="AD38">
+        <v>4</v>
+      </c>
+      <c r="AE38">
+        <v>0</v>
+      </c>
+      <c r="AF38">
+        <v>0</v>
+      </c>
+      <c r="AG38">
+        <v>11</v>
+      </c>
+      <c r="AH38">
+        <v>6</v>
+      </c>
+      <c r="AI38">
+        <v>10</v>
+      </c>
+      <c r="AJ38">
+        <v>5</v>
+      </c>
+      <c r="AK38">
+        <v>1.94</v>
+      </c>
+      <c r="AL38">
+        <v>0.63</v>
+      </c>
+      <c r="AM38">
+        <v>0.37</v>
+      </c>
+      <c r="AN38">
+        <v>0.67</v>
+      </c>
+      <c r="AO38">
+        <v>2.31</v>
+      </c>
+      <c r="AP38">
+        <v>1.31</v>
+      </c>
+      <c r="AQ38">
+        <v>2.17</v>
+      </c>
+      <c r="AR38">
+        <v>1.89</v>
+      </c>
+      <c r="AS38">
+        <v>749</v>
+      </c>
+      <c r="AT38">
+        <v>295</v>
+      </c>
+      <c r="AU38">
+        <v>137</v>
+      </c>
+      <c r="AV38">
+        <v>146</v>
+      </c>
+      <c r="AW38">
+        <v>534</v>
+      </c>
+      <c r="AX38">
+        <v>70</v>
+      </c>
+      <c r="AY38">
+        <v>22</v>
+      </c>
+      <c r="AZ38">
+        <v>20</v>
+      </c>
+      <c r="BA38">
+        <v>4</v>
+      </c>
+      <c r="BB38">
+        <v>3</v>
+      </c>
+      <c r="BC38">
+        <v>22</v>
+      </c>
+      <c r="BD38">
+        <v>21</v>
+      </c>
+      <c r="BE38">
+        <v>46</v>
+      </c>
+      <c r="BF38">
+        <v>14</v>
+      </c>
+      <c r="BG38">
+        <v>1</v>
+      </c>
+      <c r="BH38">
+        <v>4</v>
+      </c>
+      <c r="BI38" t="s">
+        <v>90</v>
+      </c>
+      <c r="BJ38" t="s">
+        <v>90</v>
+      </c>
+      <c r="BK38">
+        <v>14</v>
+      </c>
+      <c r="BL38">
+        <v>20</v>
+      </c>
+      <c r="BM38">
+        <v>9</v>
+      </c>
+      <c r="BN38">
+        <v>12</v>
+      </c>
+      <c r="BO38">
+        <v>4</v>
+      </c>
+      <c r="BP38">
+        <v>3</v>
+      </c>
+      <c r="BQ38">
+        <v>19</v>
+      </c>
+      <c r="BR38">
+        <v>43</v>
+      </c>
+      <c r="BS38">
+        <v>2</v>
+      </c>
+      <c r="BT38">
+        <v>7</v>
+      </c>
+      <c r="BU38" t="s">
+        <v>90</v>
+      </c>
+      <c r="BV38" t="s">
+        <v>90</v>
+      </c>
+      <c r="BW38">
+        <v>40</v>
+      </c>
+      <c r="BX38">
+        <v>52</v>
+      </c>
+      <c r="BY38">
+        <v>29</v>
+      </c>
+      <c r="BZ38">
+        <v>38</v>
+      </c>
+      <c r="CA38">
+        <v>11</v>
+      </c>
+      <c r="CB38">
+        <v>14</v>
+      </c>
+      <c r="CC38">
+        <v>6</v>
+      </c>
+      <c r="CD38">
+        <v>9</v>
+      </c>
+      <c r="CE38" t="s">
+        <v>90</v>
+      </c>
+      <c r="CF38" t="s">
+        <v>90</v>
+      </c>
+      <c r="CG38">
+        <v>2</v>
+      </c>
+      <c r="CH38">
+        <v>1</v>
+      </c>
+      <c r="CI38">
+        <v>0</v>
+      </c>
+      <c r="CJ38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="2:88" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B39" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="C39" t="s">
+        <v>108</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E39">
+        <v>2</v>
+      </c>
+      <c r="F39">
+        <v>2</v>
+      </c>
+      <c r="G39">
+        <v>30</v>
+      </c>
+      <c r="H39">
+        <f t="shared" si="0"/>
+        <v>70</v>
+      </c>
+      <c r="I39">
+        <v>2.37</v>
+      </c>
+      <c r="J39">
+        <v>4.96</v>
+      </c>
+      <c r="K39">
+        <v>12</v>
+      </c>
+      <c r="L39">
+        <v>30</v>
+      </c>
+      <c r="M39">
+        <v>5</v>
+      </c>
+      <c r="N39">
+        <v>10</v>
+      </c>
+      <c r="O39">
+        <v>3</v>
+      </c>
+      <c r="P39">
+        <v>7</v>
+      </c>
+      <c r="Q39">
+        <v>1</v>
+      </c>
+      <c r="R39">
+        <v>5</v>
+      </c>
+      <c r="S39">
+        <v>217</v>
+      </c>
+      <c r="T39">
+        <v>582</v>
+      </c>
+      <c r="U39">
+        <v>10</v>
+      </c>
+      <c r="V39">
+        <v>6</v>
+      </c>
+      <c r="W39">
+        <v>5</v>
+      </c>
+      <c r="X39">
+        <v>9</v>
+      </c>
+      <c r="Y39" t="s">
+        <v>90</v>
+      </c>
+      <c r="Z39" t="s">
+        <v>90</v>
+      </c>
+      <c r="AA39">
+        <v>4</v>
+      </c>
+      <c r="AB39">
+        <v>11</v>
+      </c>
+      <c r="AC39">
+        <v>3</v>
+      </c>
+      <c r="AD39">
+        <v>9</v>
+      </c>
+      <c r="AE39">
+        <v>0</v>
+      </c>
+      <c r="AF39">
+        <v>2</v>
+      </c>
+      <c r="AG39">
+        <v>10</v>
+      </c>
+      <c r="AH39">
+        <v>17</v>
+      </c>
+      <c r="AI39">
+        <v>2</v>
+      </c>
+      <c r="AJ39">
+        <v>13</v>
+      </c>
+      <c r="AK39">
+        <v>1.74</v>
+      </c>
+      <c r="AL39">
+        <v>4.2300000000000004</v>
+      </c>
+      <c r="AM39">
+        <v>0.63</v>
+      </c>
+      <c r="AN39">
+        <v>0.73</v>
+      </c>
+      <c r="AO39">
+        <v>2.37</v>
+      </c>
+      <c r="AP39">
+        <v>4.96</v>
+      </c>
+      <c r="AQ39">
+        <v>2</v>
+      </c>
+      <c r="AR39">
+        <v>4.29</v>
+      </c>
+      <c r="AS39">
+        <v>286</v>
+      </c>
+      <c r="AT39">
+        <v>649</v>
+      </c>
+      <c r="AU39">
+        <v>124</v>
+      </c>
+      <c r="AV39">
+        <v>119</v>
+      </c>
+      <c r="AW39">
+        <v>93</v>
+      </c>
+      <c r="AX39">
+        <v>463</v>
+      </c>
+      <c r="AY39">
+        <v>24</v>
+      </c>
+      <c r="AZ39">
+        <v>23</v>
+      </c>
+      <c r="BA39">
+        <v>1</v>
+      </c>
+      <c r="BB39">
+        <v>6</v>
+      </c>
+      <c r="BC39">
+        <v>14</v>
+      </c>
+      <c r="BD39">
+        <v>22</v>
+      </c>
+      <c r="BE39">
+        <v>23</v>
+      </c>
+      <c r="BF39">
+        <v>62</v>
+      </c>
+      <c r="BG39">
+        <v>1</v>
+      </c>
+      <c r="BH39">
+        <v>4</v>
+      </c>
+      <c r="BI39" t="s">
+        <v>90</v>
+      </c>
+      <c r="BJ39" t="s">
+        <v>90</v>
+      </c>
+      <c r="BK39">
+        <v>24</v>
+      </c>
+      <c r="BL39">
+        <v>13</v>
+      </c>
+      <c r="BM39">
+        <v>13</v>
+      </c>
+      <c r="BN39">
+        <v>4</v>
+      </c>
+      <c r="BO39">
+        <v>9</v>
+      </c>
+      <c r="BP39">
+        <v>3</v>
+      </c>
+      <c r="BQ39">
+        <v>36</v>
+      </c>
+      <c r="BR39">
+        <v>14</v>
+      </c>
+      <c r="BS39">
+        <v>8</v>
+      </c>
+      <c r="BT39">
+        <v>3</v>
+      </c>
+      <c r="BU39" t="s">
+        <v>90</v>
+      </c>
+      <c r="BV39" t="s">
+        <v>90</v>
+      </c>
+      <c r="BW39">
+        <v>44</v>
+      </c>
+      <c r="BX39">
+        <v>41</v>
+      </c>
+      <c r="BY39">
+        <v>38</v>
+      </c>
+      <c r="BZ39">
+        <v>34</v>
+      </c>
+      <c r="CA39">
+        <v>6</v>
+      </c>
+      <c r="CB39">
+        <v>7</v>
+      </c>
+      <c r="CC39">
+        <v>8</v>
+      </c>
+      <c r="CD39">
+        <v>11</v>
+      </c>
+      <c r="CE39" t="s">
+        <v>90</v>
+      </c>
+      <c r="CF39" t="s">
+        <v>90</v>
+      </c>
+      <c r="CG39">
+        <v>3</v>
+      </c>
+      <c r="CH39">
+        <v>0</v>
+      </c>
+      <c r="CI39">
+        <v>0</v>
+      </c>
+      <c r="CJ39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="2:88" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B40" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="C40" t="s">
+        <v>95</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="E40">
+        <v>2</v>
+      </c>
+      <c r="F40">
+        <v>3</v>
+      </c>
+      <c r="G40">
+        <v>64</v>
+      </c>
+      <c r="H40">
+        <f t="shared" si="0"/>
+        <v>36</v>
+      </c>
+      <c r="I40">
+        <v>0.93</v>
+      </c>
+      <c r="J40">
+        <v>1.28</v>
+      </c>
+      <c r="K40">
+        <v>17</v>
+      </c>
+      <c r="L40">
+        <v>15</v>
+      </c>
+      <c r="M40">
+        <v>4</v>
+      </c>
+      <c r="N40">
+        <v>4</v>
+      </c>
+      <c r="O40">
+        <v>3</v>
+      </c>
+      <c r="P40">
+        <v>3</v>
+      </c>
+      <c r="Q40">
+        <v>3</v>
+      </c>
+      <c r="R40">
+        <v>1</v>
+      </c>
+      <c r="S40">
+        <v>444</v>
+      </c>
+      <c r="T40">
+        <v>211</v>
+      </c>
+      <c r="U40">
+        <v>11</v>
+      </c>
+      <c r="V40">
+        <v>16</v>
+      </c>
+      <c r="W40">
+        <v>7</v>
+      </c>
+      <c r="X40">
+        <v>3</v>
+      </c>
+      <c r="Y40" t="s">
+        <v>90</v>
+      </c>
+      <c r="Z40" t="s">
+        <v>90</v>
+      </c>
+      <c r="AA40">
+        <v>5</v>
+      </c>
+      <c r="AB40">
+        <v>7</v>
+      </c>
+      <c r="AC40">
+        <v>8</v>
+      </c>
+      <c r="AD40">
+        <v>4</v>
+      </c>
+      <c r="AE40">
+        <v>0</v>
+      </c>
+      <c r="AF40">
+        <v>1</v>
+      </c>
+      <c r="AG40">
+        <v>9</v>
+      </c>
+      <c r="AH40">
+        <v>10</v>
+      </c>
+      <c r="AI40">
+        <v>8</v>
+      </c>
+      <c r="AJ40">
+        <v>5</v>
+      </c>
+      <c r="AK40">
+        <v>0.73</v>
+      </c>
+      <c r="AL40">
+        <v>0.62</v>
+      </c>
+      <c r="AM40">
+        <v>0.2</v>
+      </c>
+      <c r="AN40">
+        <v>0.66</v>
+      </c>
+      <c r="AO40">
+        <v>0.93</v>
+      </c>
+      <c r="AP40">
+        <v>1.28</v>
+      </c>
+      <c r="AQ40">
+        <v>0.68</v>
+      </c>
+      <c r="AR40">
+        <v>1.66</v>
+      </c>
+      <c r="AS40">
+        <v>545</v>
+      </c>
+      <c r="AT40">
+        <v>306</v>
+      </c>
+      <c r="AU40">
+        <v>188</v>
+      </c>
+      <c r="AV40">
+        <v>104</v>
+      </c>
+      <c r="AW40">
+        <v>256</v>
+      </c>
+      <c r="AX40">
+        <v>107</v>
+      </c>
+      <c r="AY40">
+        <v>20</v>
+      </c>
+      <c r="AZ40">
+        <v>25</v>
+      </c>
+      <c r="BA40">
+        <v>7</v>
+      </c>
+      <c r="BB40">
+        <v>5</v>
+      </c>
+      <c r="BC40">
+        <v>25</v>
+      </c>
+      <c r="BD40">
+        <v>17</v>
+      </c>
+      <c r="BE40">
+        <v>41</v>
+      </c>
+      <c r="BF40">
+        <v>19</v>
+      </c>
+      <c r="BG40">
+        <v>3</v>
+      </c>
+      <c r="BH40">
+        <v>1</v>
+      </c>
+      <c r="BI40" t="s">
+        <v>90</v>
+      </c>
+      <c r="BJ40" t="s">
+        <v>90</v>
+      </c>
+      <c r="BK40">
+        <v>13</v>
+      </c>
+      <c r="BL40">
+        <v>18</v>
+      </c>
+      <c r="BM40">
+        <v>15</v>
+      </c>
+      <c r="BN40">
+        <v>12</v>
+      </c>
+      <c r="BO40">
+        <v>4</v>
+      </c>
+      <c r="BP40">
+        <v>8</v>
+      </c>
+      <c r="BQ40">
+        <v>25</v>
+      </c>
+      <c r="BR40">
+        <v>40</v>
+      </c>
+      <c r="BS40">
+        <v>1</v>
+      </c>
+      <c r="BT40">
+        <v>3</v>
+      </c>
+      <c r="BU40" t="s">
+        <v>90</v>
+      </c>
+      <c r="BV40" t="s">
+        <v>90</v>
+      </c>
+      <c r="BW40">
+        <v>65</v>
+      </c>
+      <c r="BX40">
+        <v>49</v>
+      </c>
+      <c r="BY40">
+        <v>37</v>
+      </c>
+      <c r="BZ40">
+        <v>32</v>
+      </c>
+      <c r="CA40">
+        <v>28</v>
+      </c>
+      <c r="CB40">
+        <v>17</v>
+      </c>
+      <c r="CC40">
+        <v>10</v>
+      </c>
+      <c r="CD40">
+        <v>4</v>
+      </c>
+      <c r="CE40" t="s">
+        <v>90</v>
+      </c>
+      <c r="CF40" t="s">
+        <v>90</v>
+      </c>
+      <c r="CG40">
+        <v>1</v>
+      </c>
+      <c r="CH40">
+        <v>0</v>
+      </c>
+      <c r="CI40">
+        <v>1</v>
+      </c>
+      <c r="CJ40">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="2:88" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B41" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="C41" t="s">
+        <v>96</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="E41">
+        <v>3</v>
+      </c>
+      <c r="F41">
+        <v>4</v>
+      </c>
+      <c r="G41">
+        <v>47</v>
+      </c>
+      <c r="H41">
+        <f t="shared" si="0"/>
+        <v>53</v>
+      </c>
+      <c r="I41">
+        <v>2.87</v>
+      </c>
+      <c r="J41">
+        <v>1.69</v>
+      </c>
+      <c r="K41">
+        <v>23</v>
+      </c>
+      <c r="L41">
+        <v>16</v>
+      </c>
+      <c r="M41">
+        <v>5</v>
+      </c>
+      <c r="N41">
+        <v>7</v>
+      </c>
+      <c r="O41">
+        <v>2</v>
+      </c>
+      <c r="P41">
+        <v>4</v>
+      </c>
+      <c r="Q41">
+        <v>1</v>
+      </c>
+      <c r="R41">
+        <v>2</v>
+      </c>
+      <c r="S41">
+        <v>367</v>
+      </c>
+      <c r="T41">
+        <v>433</v>
+      </c>
+      <c r="U41">
+        <v>11</v>
+      </c>
+      <c r="V41">
+        <v>10</v>
+      </c>
+      <c r="W41">
+        <v>4</v>
+      </c>
+      <c r="X41">
+        <v>3</v>
+      </c>
+      <c r="Y41" t="s">
+        <v>90</v>
+      </c>
+      <c r="Z41" t="s">
+        <v>90</v>
+      </c>
+      <c r="AA41">
+        <v>11</v>
+      </c>
+      <c r="AB41">
+        <v>6</v>
+      </c>
+      <c r="AC41">
+        <v>7</v>
+      </c>
+      <c r="AD41">
+        <v>3</v>
+      </c>
+      <c r="AE41">
+        <v>0</v>
+      </c>
+      <c r="AF41">
+        <v>0</v>
+      </c>
+      <c r="AG41">
+        <v>17</v>
+      </c>
+      <c r="AH41">
+        <v>12</v>
+      </c>
+      <c r="AI41">
+        <v>6</v>
+      </c>
+      <c r="AJ41">
+        <v>4</v>
+      </c>
+      <c r="AK41">
+        <v>1.24</v>
+      </c>
+      <c r="AL41">
+        <v>1.54</v>
+      </c>
+      <c r="AM41">
+        <v>1.63</v>
+      </c>
+      <c r="AN41">
+        <v>0.15</v>
+      </c>
+      <c r="AO41">
+        <v>2.87</v>
+      </c>
+      <c r="AP41">
+        <v>1.69</v>
+      </c>
+      <c r="AQ41">
+        <v>1.39</v>
+      </c>
+      <c r="AR41">
+        <v>2.5099999999999998</v>
+      </c>
+      <c r="AS41">
+        <v>442</v>
+      </c>
+      <c r="AT41">
+        <v>508</v>
+      </c>
+      <c r="AU41">
+        <v>176</v>
+      </c>
+      <c r="AV41">
+        <v>215</v>
+      </c>
+      <c r="AW41">
+        <v>191</v>
+      </c>
+      <c r="AX41">
+        <v>218</v>
+      </c>
+      <c r="AY41">
+        <v>16</v>
+      </c>
+      <c r="AZ41">
+        <v>22</v>
+      </c>
+      <c r="BA41">
+        <v>13</v>
+      </c>
+      <c r="BB41">
+        <v>2</v>
+      </c>
+      <c r="BC41">
+        <v>13</v>
+      </c>
+      <c r="BD41">
+        <v>20</v>
+      </c>
+      <c r="BE41">
+        <v>33</v>
+      </c>
+      <c r="BF41">
+        <v>26</v>
+      </c>
+      <c r="BG41">
+        <v>0</v>
+      </c>
+      <c r="BH41">
+        <v>1</v>
+      </c>
+      <c r="BI41" t="s">
+        <v>90</v>
+      </c>
+      <c r="BJ41" t="s">
+        <v>90</v>
+      </c>
+      <c r="BK41">
+        <v>17</v>
+      </c>
+      <c r="BL41">
+        <v>16</v>
+      </c>
+      <c r="BM41">
+        <v>10</v>
+      </c>
+      <c r="BN41">
+        <v>10</v>
+      </c>
+      <c r="BO41">
+        <v>3</v>
+      </c>
+      <c r="BP41">
+        <v>8</v>
+      </c>
+      <c r="BQ41">
+        <v>18</v>
+      </c>
+      <c r="BR41">
+        <v>20</v>
+      </c>
+      <c r="BS41">
+        <v>3</v>
+      </c>
+      <c r="BT41">
+        <v>1</v>
+      </c>
+      <c r="BU41" t="s">
+        <v>90</v>
+      </c>
+      <c r="BV41" t="s">
+        <v>90</v>
+      </c>
+      <c r="BW41">
+        <v>43</v>
+      </c>
+      <c r="BX41">
+        <v>37</v>
+      </c>
+      <c r="BY41">
+        <v>30</v>
+      </c>
+      <c r="BZ41">
+        <v>31</v>
+      </c>
+      <c r="CA41">
+        <v>13</v>
+      </c>
+      <c r="CB41">
+        <v>6</v>
+      </c>
+      <c r="CC41">
+        <v>2</v>
+      </c>
+      <c r="CD41">
+        <v>4</v>
+      </c>
+      <c r="CE41" t="s">
+        <v>90</v>
+      </c>
+      <c r="CF41" t="s">
+        <v>90</v>
+      </c>
+      <c r="CG41">
+        <v>3</v>
+      </c>
+      <c r="CH41">
+        <v>1</v>
+      </c>
+      <c r="CI41">
+        <v>0</v>
+      </c>
+      <c r="CJ41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="2:88" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B42" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="C42" t="s">
+        <v>97</v>
+      </c>
+      <c r="D42" t="s">
+        <v>88</v>
+      </c>
+      <c r="E42">
+        <v>0</v>
+      </c>
+      <c r="F42">
+        <v>2</v>
+      </c>
+      <c r="G42">
+        <v>52</v>
+      </c>
+      <c r="H42">
+        <f t="shared" si="0"/>
+        <v>48</v>
+      </c>
+      <c r="I42">
+        <v>1.96</v>
+      </c>
+      <c r="J42">
+        <v>2.4700000000000002</v>
+      </c>
+      <c r="K42">
+        <v>24</v>
+      </c>
+      <c r="L42">
+        <v>18</v>
+      </c>
+      <c r="M42">
+        <v>6</v>
+      </c>
+      <c r="N42">
+        <v>8</v>
+      </c>
+      <c r="O42">
+        <v>4</v>
+      </c>
+      <c r="P42">
+        <v>6</v>
+      </c>
+      <c r="Q42">
+        <v>4</v>
+      </c>
+      <c r="R42">
+        <v>5</v>
+      </c>
+      <c r="S42">
+        <v>400</v>
+      </c>
+      <c r="T42">
+        <v>358</v>
+      </c>
+      <c r="U42">
+        <v>10</v>
+      </c>
+      <c r="V42">
+        <v>11</v>
+      </c>
+      <c r="W42">
+        <v>7</v>
+      </c>
+      <c r="X42">
+        <v>5</v>
+      </c>
+      <c r="Y42" t="s">
+        <v>90</v>
+      </c>
+      <c r="Z42" t="s">
+        <v>90</v>
+      </c>
+      <c r="AA42">
+        <v>10</v>
+      </c>
+      <c r="AB42">
+        <v>5</v>
+      </c>
+      <c r="AC42">
+        <v>8</v>
+      </c>
+      <c r="AD42">
+        <v>5</v>
+      </c>
+      <c r="AE42">
+        <v>0</v>
+      </c>
+      <c r="AF42">
+        <v>1</v>
+      </c>
+      <c r="AG42">
+        <v>16</v>
+      </c>
+      <c r="AH42">
+        <v>16</v>
+      </c>
+      <c r="AI42">
+        <v>8</v>
+      </c>
+      <c r="AJ42">
+        <v>2</v>
+      </c>
+      <c r="AK42">
+        <v>1.51</v>
+      </c>
+      <c r="AL42">
+        <v>2.02</v>
+      </c>
+      <c r="AM42">
+        <v>0.45</v>
+      </c>
+      <c r="AN42">
+        <v>0.46</v>
+      </c>
+      <c r="AO42">
+        <v>1.96</v>
+      </c>
+      <c r="AP42">
+        <v>2.4700000000000002</v>
+      </c>
+      <c r="AQ42">
+        <v>0.4</v>
+      </c>
+      <c r="AR42">
+        <v>1.85</v>
+      </c>
+      <c r="AS42">
+        <v>489</v>
+      </c>
+      <c r="AT42">
+        <v>458</v>
+      </c>
+      <c r="AU42">
+        <v>209</v>
+      </c>
+      <c r="AV42">
+        <v>217</v>
+      </c>
+      <c r="AW42">
+        <v>191</v>
+      </c>
+      <c r="AX42">
+        <v>141</v>
+      </c>
+      <c r="AY42">
+        <v>22</v>
+      </c>
+      <c r="AZ42">
+        <v>28</v>
+      </c>
+      <c r="BA42">
+        <v>8</v>
+      </c>
+      <c r="BB42">
+        <v>4</v>
+      </c>
+      <c r="BC42">
+        <v>19</v>
+      </c>
+      <c r="BD42">
+        <v>15</v>
+      </c>
+      <c r="BE42">
+        <v>36</v>
+      </c>
+      <c r="BF42">
+        <v>34</v>
+      </c>
+      <c r="BG42">
+        <v>1</v>
+      </c>
+      <c r="BH42">
+        <v>1</v>
+      </c>
+      <c r="BI42" t="s">
+        <v>90</v>
+      </c>
+      <c r="BJ42" t="s">
+        <v>90</v>
+      </c>
+      <c r="BK42">
+        <v>23</v>
+      </c>
+      <c r="BL42">
+        <v>21</v>
+      </c>
+      <c r="BM42">
+        <v>15</v>
+      </c>
+      <c r="BN42">
+        <v>10</v>
+      </c>
+      <c r="BO42">
+        <v>6</v>
+      </c>
+      <c r="BP42">
+        <v>10</v>
+      </c>
+      <c r="BQ42">
+        <v>15</v>
+      </c>
+      <c r="BR42">
+        <v>41</v>
+      </c>
+      <c r="BS42">
+        <v>5</v>
+      </c>
+      <c r="BT42">
+        <v>4</v>
+      </c>
+      <c r="BU42" t="s">
+        <v>90</v>
+      </c>
+      <c r="BV42" t="s">
+        <v>90</v>
+      </c>
+      <c r="BW42">
+        <v>64</v>
+      </c>
+      <c r="BX42">
+        <v>62</v>
+      </c>
+      <c r="BY42">
+        <v>45</v>
+      </c>
+      <c r="BZ42">
+        <v>38</v>
+      </c>
+      <c r="CA42">
+        <v>19</v>
+      </c>
+      <c r="CB42">
+        <v>24</v>
+      </c>
+      <c r="CC42">
+        <v>11</v>
+      </c>
+      <c r="CD42">
+        <v>7</v>
+      </c>
+      <c r="CE42" t="s">
+        <v>90</v>
+      </c>
+      <c r="CF42" t="s">
+        <v>90</v>
+      </c>
+      <c r="CG42">
+        <v>1</v>
+      </c>
+      <c r="CH42">
+        <v>0</v>
+      </c>
+      <c r="CI42">
+        <v>0</v>
+      </c>
+      <c r="CJ42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="2:88" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B43" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="C43" t="s">
+        <v>100</v>
+      </c>
+      <c r="D43" t="s">
+        <v>92</v>
+      </c>
+      <c r="E43">
+        <v>1</v>
+      </c>
+      <c r="F43">
+        <v>0</v>
+      </c>
+      <c r="G43">
+        <v>43</v>
+      </c>
+      <c r="H43">
+        <f t="shared" si="0"/>
+        <v>57</v>
+      </c>
+      <c r="I43">
+        <v>1.1299999999999999</v>
+      </c>
+      <c r="J43">
+        <v>0.24</v>
+      </c>
+      <c r="K43">
+        <v>19</v>
+      </c>
+      <c r="L43">
+        <v>7</v>
+      </c>
+      <c r="M43">
+        <v>6</v>
+      </c>
+      <c r="N43">
+        <v>2</v>
+      </c>
+      <c r="O43">
+        <v>0</v>
+      </c>
+      <c r="P43">
+        <v>0</v>
+      </c>
+      <c r="Q43">
+        <v>0</v>
+      </c>
+      <c r="R43">
+        <v>0</v>
+      </c>
+      <c r="S43">
+        <v>252</v>
+      </c>
+      <c r="T43">
+        <v>368</v>
+      </c>
+      <c r="U43">
+        <v>14</v>
+      </c>
+      <c r="V43">
+        <v>9</v>
+      </c>
+      <c r="W43">
+        <v>7</v>
+      </c>
+      <c r="X43">
+        <v>3</v>
+      </c>
+      <c r="Y43" t="s">
+        <v>90</v>
+      </c>
+      <c r="Z43" t="s">
+        <v>90</v>
+      </c>
+      <c r="AA43">
+        <v>7</v>
+      </c>
+      <c r="AB43">
+        <v>5</v>
+      </c>
+      <c r="AC43">
+        <v>6</v>
+      </c>
+      <c r="AD43">
+        <v>0</v>
+      </c>
+      <c r="AE43">
+        <v>0</v>
+      </c>
+      <c r="AF43">
+        <v>2</v>
+      </c>
+      <c r="AG43">
+        <v>13</v>
+      </c>
+      <c r="AH43">
+        <v>6</v>
+      </c>
+      <c r="AI43">
+        <v>6</v>
+      </c>
+      <c r="AJ43">
+        <v>1</v>
+      </c>
+      <c r="AK43">
+        <v>0.73</v>
+      </c>
+      <c r="AL43">
+        <v>0.08</v>
+      </c>
+      <c r="AM43">
+        <v>0.41</v>
+      </c>
+      <c r="AN43">
+        <v>0.16</v>
+      </c>
+      <c r="AO43">
+        <v>1.1299999999999999</v>
+      </c>
+      <c r="AP43">
+        <v>0.24</v>
+      </c>
+      <c r="AQ43">
+        <v>1.0900000000000001</v>
+      </c>
+      <c r="AR43">
+        <v>0.15</v>
+      </c>
+      <c r="AS43">
+        <v>326</v>
+      </c>
+      <c r="AT43">
+        <v>452</v>
+      </c>
+      <c r="AU43">
+        <v>142</v>
+      </c>
+      <c r="AV43">
+        <v>232</v>
+      </c>
+      <c r="AW43">
+        <v>110</v>
+      </c>
+      <c r="AX43">
+        <v>136</v>
+      </c>
+      <c r="AY43">
+        <v>23</v>
+      </c>
+      <c r="AZ43">
+        <v>32</v>
+      </c>
+      <c r="BA43">
+        <v>8</v>
+      </c>
+      <c r="BB43">
+        <v>5</v>
+      </c>
+      <c r="BC43">
+        <v>24</v>
+      </c>
+      <c r="BD43">
+        <v>28</v>
+      </c>
+      <c r="BE43">
+        <v>23</v>
+      </c>
+      <c r="BF43">
+        <v>22</v>
+      </c>
+      <c r="BG43">
+        <v>3</v>
+      </c>
+      <c r="BH43">
+        <v>7</v>
+      </c>
+      <c r="BI43" t="s">
+        <v>90</v>
+      </c>
+      <c r="BJ43" t="s">
+        <v>90</v>
+      </c>
+      <c r="BK43">
+        <v>16</v>
+      </c>
+      <c r="BL43">
+        <v>12</v>
+      </c>
+      <c r="BM43">
+        <v>17</v>
+      </c>
+      <c r="BN43">
+        <v>7</v>
+      </c>
+      <c r="BO43">
+        <v>0</v>
+      </c>
+      <c r="BP43">
+        <v>6</v>
+      </c>
+      <c r="BQ43">
+        <v>29</v>
+      </c>
+      <c r="BR43">
+        <v>28</v>
+      </c>
+      <c r="BS43">
+        <v>2</v>
+      </c>
+      <c r="BT43">
+        <v>5</v>
+      </c>
+      <c r="BU43" t="s">
+        <v>90</v>
+      </c>
+      <c r="BV43" t="s">
+        <v>90</v>
+      </c>
+      <c r="BW43">
+        <v>49</v>
+      </c>
+      <c r="BX43">
+        <v>51</v>
+      </c>
+      <c r="BY43">
+        <v>31</v>
+      </c>
+      <c r="BZ43">
+        <v>30</v>
+      </c>
+      <c r="CA43">
+        <v>18</v>
+      </c>
+      <c r="CB43">
+        <v>21</v>
+      </c>
+      <c r="CC43">
+        <v>7</v>
+      </c>
+      <c r="CD43">
+        <v>5</v>
+      </c>
+      <c r="CE43" t="s">
+        <v>90</v>
+      </c>
+      <c r="CF43" t="s">
+        <v>90</v>
+      </c>
+      <c r="CG43">
+        <v>2</v>
+      </c>
+      <c r="CH43">
+        <v>1</v>
+      </c>
+      <c r="CI43">
+        <v>0</v>
+      </c>
+      <c r="CJ43">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="2:88" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B44" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C44" t="s">
+        <v>98</v>
+      </c>
+      <c r="D44" t="s">
+        <v>101</v>
+      </c>
+      <c r="E44">
+        <v>6</v>
+      </c>
+      <c r="F44">
+        <v>0</v>
+      </c>
+      <c r="G44">
+        <v>47</v>
+      </c>
+      <c r="H44">
+        <f t="shared" si="0"/>
+        <v>53</v>
+      </c>
+      <c r="I44">
+        <v>4.03</v>
+      </c>
+      <c r="J44">
+        <v>1.46</v>
+      </c>
+      <c r="K44">
+        <v>20</v>
+      </c>
+      <c r="L44">
+        <v>18</v>
+      </c>
+      <c r="M44">
+        <v>10</v>
+      </c>
+      <c r="N44">
+        <v>9</v>
+      </c>
+      <c r="O44">
+        <v>8</v>
+      </c>
+      <c r="P44">
+        <v>5</v>
+      </c>
+      <c r="Q44">
+        <v>3</v>
+      </c>
+      <c r="R44">
+        <v>5</v>
+      </c>
+      <c r="S44">
+        <v>376</v>
+      </c>
+      <c r="T44">
+        <v>423</v>
+      </c>
+      <c r="U44">
+        <v>16</v>
+      </c>
+      <c r="V44">
+        <v>13</v>
+      </c>
+      <c r="W44">
+        <v>3</v>
+      </c>
+      <c r="X44">
+        <v>6</v>
+      </c>
+      <c r="Y44" t="s">
+        <v>90</v>
+      </c>
+      <c r="Z44" t="s">
+        <v>90</v>
+      </c>
+      <c r="AA44">
+        <v>5</v>
+      </c>
+      <c r="AB44">
+        <v>5</v>
+      </c>
+      <c r="AC44">
+        <v>5</v>
+      </c>
+      <c r="AD44">
+        <v>4</v>
+      </c>
+      <c r="AE44">
+        <v>0</v>
+      </c>
+      <c r="AF44">
+        <v>0</v>
+      </c>
+      <c r="AG44">
+        <v>18</v>
+      </c>
+      <c r="AH44">
+        <v>16</v>
+      </c>
+      <c r="AI44">
+        <v>2</v>
+      </c>
+      <c r="AJ44">
+        <v>2</v>
+      </c>
+      <c r="AK44">
+        <v>3.05</v>
+      </c>
+      <c r="AL44">
+        <v>1.17</v>
+      </c>
+      <c r="AM44">
+        <v>0.97</v>
+      </c>
+      <c r="AN44">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="AO44">
+        <v>4.03</v>
+      </c>
+      <c r="AP44">
+        <v>1.46</v>
+      </c>
+      <c r="AQ44">
+        <v>4.9800000000000004</v>
+      </c>
+      <c r="AR44">
+        <v>2.33</v>
+      </c>
+      <c r="AS44">
+        <v>434</v>
+      </c>
+      <c r="AT44">
+        <v>486</v>
+      </c>
+      <c r="AU44">
+        <v>256</v>
+      </c>
+      <c r="AV44">
+        <v>218</v>
+      </c>
+      <c r="AW44">
+        <v>120</v>
+      </c>
+      <c r="AX44">
+        <v>205</v>
+      </c>
+      <c r="AY44">
+        <v>25</v>
+      </c>
+      <c r="AZ44">
+        <v>23</v>
+      </c>
+      <c r="BA44">
+        <v>5</v>
+      </c>
+      <c r="BB44">
+        <v>6</v>
+      </c>
+      <c r="BC44">
+        <v>17</v>
+      </c>
+      <c r="BD44">
+        <v>15</v>
+      </c>
+      <c r="BE44">
+        <v>37</v>
+      </c>
+      <c r="BF44">
+        <v>32</v>
+      </c>
+      <c r="BG44">
+        <v>1</v>
+      </c>
+      <c r="BH44">
+        <v>2</v>
+      </c>
+      <c r="BI44" t="s">
+        <v>90</v>
+      </c>
+      <c r="BJ44" t="s">
+        <v>90</v>
+      </c>
+      <c r="BK44">
+        <v>24</v>
+      </c>
+      <c r="BL44">
+        <v>20</v>
+      </c>
+      <c r="BM44">
+        <v>8</v>
+      </c>
+      <c r="BN44">
+        <v>11</v>
+      </c>
+      <c r="BO44">
+        <v>4</v>
+      </c>
+      <c r="BP44">
+        <v>4</v>
+      </c>
+      <c r="BQ44">
+        <v>26</v>
+      </c>
+      <c r="BR44">
+        <v>17</v>
+      </c>
+      <c r="BS44">
+        <v>9</v>
+      </c>
+      <c r="BT44">
+        <v>4</v>
+      </c>
+      <c r="BU44" t="s">
+        <v>90</v>
+      </c>
+      <c r="BV44" t="s">
+        <v>90</v>
+      </c>
+      <c r="BW44">
+        <v>57</v>
+      </c>
+      <c r="BX44">
+        <v>53</v>
+      </c>
+      <c r="BY44">
+        <v>46</v>
+      </c>
+      <c r="BZ44">
+        <v>43</v>
+      </c>
+      <c r="CA44">
+        <v>11</v>
+      </c>
+      <c r="CB44">
+        <v>10</v>
+      </c>
+      <c r="CC44">
+        <v>10</v>
+      </c>
+      <c r="CD44">
+        <v>7</v>
+      </c>
+      <c r="CE44" t="s">
+        <v>90</v>
+      </c>
+      <c r="CF44" t="s">
+        <v>90</v>
+      </c>
+      <c r="CG44">
+        <v>1</v>
+      </c>
+      <c r="CH44">
+        <v>3</v>
+      </c>
+      <c r="CI44">
+        <v>0</v>
+      </c>
+      <c r="CJ44">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Oct 16, 2026, 7:20 PM
</commit_message>
<xml_diff>
--- a/Bundesliga 26-27.xlsx
+++ b/Bundesliga 26-27.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kuba\Desktop\analityczka\26-27\Ekstraklasa 26-27\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3843870E-5701-4DD8-8438-1571AF6FAF51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{78DAC283-4B1C-4DF4-A956-DC2F011A8189}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{723BE2C8-720D-41E0-A496-B3B96A8488E1}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="560" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="582" uniqueCount="131">
   <si>
     <t>date</t>
   </si>
@@ -426,6 +426,12 @@
   </si>
   <si>
     <t>Sat 10 October, 18:30</t>
+  </si>
+  <si>
+    <t>Sun 11 October, 15:30</t>
+  </si>
+  <si>
+    <t>Sun 11 October, 17:30</t>
   </si>
 </sst>
 </file>
@@ -843,7 +849,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9ED51FE2-0441-4690-9385-28E7CF18BF79}">
-  <dimension ref="B1:CJ44"/>
+  <dimension ref="B1:CJ46"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="17.7109375" customWidth="1"/>
@@ -1164,7 +1170,7 @@
         <v>59</v>
       </c>
       <c r="H2">
-        <f t="shared" ref="H2:H44" si="0">100-G2</f>
+        <f t="shared" ref="H2:H46" si="0">100-G2</f>
         <v>41</v>
       </c>
       <c r="I2">
@@ -12493,6 +12499,534 @@
         <v>0</v>
       </c>
       <c r="CJ44">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="2:88" ht="30" x14ac:dyDescent="0.25">
+      <c r="B45" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="D45" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="E45">
+        <v>2</v>
+      </c>
+      <c r="F45">
+        <v>1</v>
+      </c>
+      <c r="G45">
+        <v>48</v>
+      </c>
+      <c r="H45">
+        <f t="shared" si="0"/>
+        <v>52</v>
+      </c>
+      <c r="I45">
+        <v>1.32</v>
+      </c>
+      <c r="J45">
+        <v>1.17</v>
+      </c>
+      <c r="K45">
+        <v>19</v>
+      </c>
+      <c r="L45">
+        <v>16</v>
+      </c>
+      <c r="M45">
+        <v>7</v>
+      </c>
+      <c r="N45">
+        <v>7</v>
+      </c>
+      <c r="O45">
+        <v>2</v>
+      </c>
+      <c r="P45">
+        <v>2</v>
+      </c>
+      <c r="Q45">
+        <v>2</v>
+      </c>
+      <c r="R45">
+        <v>1</v>
+      </c>
+      <c r="S45">
+        <v>312</v>
+      </c>
+      <c r="T45">
+        <v>339</v>
+      </c>
+      <c r="U45">
+        <v>8</v>
+      </c>
+      <c r="V45">
+        <v>17</v>
+      </c>
+      <c r="W45">
+        <v>6</v>
+      </c>
+      <c r="X45">
+        <v>6</v>
+      </c>
+      <c r="Y45" t="s">
+        <v>90</v>
+      </c>
+      <c r="Z45" t="s">
+        <v>90</v>
+      </c>
+      <c r="AA45">
+        <v>10</v>
+      </c>
+      <c r="AB45">
+        <v>4</v>
+      </c>
+      <c r="AC45">
+        <v>2</v>
+      </c>
+      <c r="AD45">
+        <v>5</v>
+      </c>
+      <c r="AE45">
+        <v>0</v>
+      </c>
+      <c r="AF45">
+        <v>0</v>
+      </c>
+      <c r="AG45">
+        <v>13</v>
+      </c>
+      <c r="AH45">
+        <v>7</v>
+      </c>
+      <c r="AI45">
+        <v>6</v>
+      </c>
+      <c r="AJ45">
+        <v>9</v>
+      </c>
+      <c r="AK45">
+        <v>0.9</v>
+      </c>
+      <c r="AL45">
+        <v>0.96</v>
+      </c>
+      <c r="AM45">
+        <v>0.42</v>
+      </c>
+      <c r="AN45">
+        <v>0.21</v>
+      </c>
+      <c r="AO45">
+        <v>1.32</v>
+      </c>
+      <c r="AP45">
+        <v>1.17</v>
+      </c>
+      <c r="AQ45">
+        <v>1.39</v>
+      </c>
+      <c r="AR45">
+        <v>1.77</v>
+      </c>
+      <c r="AS45">
+        <v>391</v>
+      </c>
+      <c r="AT45">
+        <v>422</v>
+      </c>
+      <c r="AU45">
+        <v>184</v>
+      </c>
+      <c r="AV45">
+        <v>159</v>
+      </c>
+      <c r="AW45">
+        <v>128</v>
+      </c>
+      <c r="AX45">
+        <v>180</v>
+      </c>
+      <c r="AY45">
+        <v>22</v>
+      </c>
+      <c r="AZ45">
+        <v>22</v>
+      </c>
+      <c r="BA45">
+        <v>5</v>
+      </c>
+      <c r="BB45">
+        <v>3</v>
+      </c>
+      <c r="BC45">
+        <v>14</v>
+      </c>
+      <c r="BD45">
+        <v>20</v>
+      </c>
+      <c r="BE45">
+        <v>28</v>
+      </c>
+      <c r="BF45">
+        <v>26</v>
+      </c>
+      <c r="BG45">
+        <v>1</v>
+      </c>
+      <c r="BH45">
+        <v>1</v>
+      </c>
+      <c r="BI45" t="s">
+        <v>90</v>
+      </c>
+      <c r="BJ45" t="s">
+        <v>90</v>
+      </c>
+      <c r="BK45">
+        <v>22</v>
+      </c>
+      <c r="BL45">
+        <v>9</v>
+      </c>
+      <c r="BM45">
+        <v>12</v>
+      </c>
+      <c r="BN45">
+        <v>4</v>
+      </c>
+      <c r="BO45">
+        <v>5</v>
+      </c>
+      <c r="BP45">
+        <v>2</v>
+      </c>
+      <c r="BQ45">
+        <v>34</v>
+      </c>
+      <c r="BR45">
+        <v>23</v>
+      </c>
+      <c r="BS45">
+        <v>6</v>
+      </c>
+      <c r="BT45">
+        <v>5</v>
+      </c>
+      <c r="BU45" t="s">
+        <v>90</v>
+      </c>
+      <c r="BV45" t="s">
+        <v>90</v>
+      </c>
+      <c r="BW45">
+        <v>65</v>
+      </c>
+      <c r="BX45">
+        <v>41</v>
+      </c>
+      <c r="BY45">
+        <v>48</v>
+      </c>
+      <c r="BZ45">
+        <v>23</v>
+      </c>
+      <c r="CA45">
+        <v>17</v>
+      </c>
+      <c r="CB45">
+        <v>18</v>
+      </c>
+      <c r="CC45">
+        <v>9</v>
+      </c>
+      <c r="CD45">
+        <v>6</v>
+      </c>
+      <c r="CE45" t="s">
+        <v>90</v>
+      </c>
+      <c r="CF45" t="s">
+        <v>90</v>
+      </c>
+      <c r="CG45">
+        <v>1</v>
+      </c>
+      <c r="CH45">
+        <v>3</v>
+      </c>
+      <c r="CI45">
+        <v>0</v>
+      </c>
+      <c r="CJ45">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="2:88" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B46" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="C46" t="s">
+        <v>106</v>
+      </c>
+      <c r="D46" t="s">
+        <v>109</v>
+      </c>
+      <c r="E46">
+        <v>2</v>
+      </c>
+      <c r="F46">
+        <v>1</v>
+      </c>
+      <c r="G46">
+        <v>51</v>
+      </c>
+      <c r="H46">
+        <f t="shared" si="0"/>
+        <v>49</v>
+      </c>
+      <c r="I46">
+        <v>1.1499999999999999</v>
+      </c>
+      <c r="J46">
+        <v>0.32</v>
+      </c>
+      <c r="K46">
+        <v>10</v>
+      </c>
+      <c r="L46">
+        <v>5</v>
+      </c>
+      <c r="M46">
+        <v>4</v>
+      </c>
+      <c r="N46">
+        <v>1</v>
+      </c>
+      <c r="O46">
+        <v>5</v>
+      </c>
+      <c r="P46">
+        <v>0</v>
+      </c>
+      <c r="Q46">
+        <v>3</v>
+      </c>
+      <c r="R46">
+        <v>0</v>
+      </c>
+      <c r="S46">
+        <v>334</v>
+      </c>
+      <c r="T46">
+        <v>328</v>
+      </c>
+      <c r="U46">
+        <v>11</v>
+      </c>
+      <c r="V46">
+        <v>13</v>
+      </c>
+      <c r="W46">
+        <v>7</v>
+      </c>
+      <c r="X46">
+        <v>2</v>
+      </c>
+      <c r="Y46" t="s">
+        <v>90</v>
+      </c>
+      <c r="Z46" t="s">
+        <v>90</v>
+      </c>
+      <c r="AA46">
+        <v>3</v>
+      </c>
+      <c r="AB46">
+        <v>1</v>
+      </c>
+      <c r="AC46">
+        <v>3</v>
+      </c>
+      <c r="AD46">
+        <v>3</v>
+      </c>
+      <c r="AE46">
+        <v>0</v>
+      </c>
+      <c r="AF46">
+        <v>1</v>
+      </c>
+      <c r="AG46">
+        <v>7</v>
+      </c>
+      <c r="AH46">
+        <v>5</v>
+      </c>
+      <c r="AI46">
+        <v>3</v>
+      </c>
+      <c r="AJ46">
+        <v>0</v>
+      </c>
+      <c r="AK46">
+        <v>0.67</v>
+      </c>
+      <c r="AL46">
+        <v>0.09</v>
+      </c>
+      <c r="AM46">
+        <v>0.48</v>
+      </c>
+      <c r="AN46">
+        <v>0.23</v>
+      </c>
+      <c r="AO46">
+        <v>1.1499999999999999</v>
+      </c>
+      <c r="AP46">
+        <v>0.32</v>
+      </c>
+      <c r="AQ46">
+        <v>1.37</v>
+      </c>
+      <c r="AR46">
+        <v>0.7</v>
+      </c>
+      <c r="AS46">
+        <v>427</v>
+      </c>
+      <c r="AT46">
+        <v>421</v>
+      </c>
+      <c r="AU46">
+        <v>230</v>
+      </c>
+      <c r="AV46">
+        <v>203</v>
+      </c>
+      <c r="AW46">
+        <v>104</v>
+      </c>
+      <c r="AX46">
+        <v>125</v>
+      </c>
+      <c r="AY46">
+        <v>26</v>
+      </c>
+      <c r="AZ46">
+        <v>34</v>
+      </c>
+      <c r="BA46">
+        <v>3</v>
+      </c>
+      <c r="BB46">
+        <v>3</v>
+      </c>
+      <c r="BC46">
+        <v>24</v>
+      </c>
+      <c r="BD46">
+        <v>16</v>
+      </c>
+      <c r="BE46">
+        <v>16</v>
+      </c>
+      <c r="BF46">
+        <v>17</v>
+      </c>
+      <c r="BG46">
+        <v>0</v>
+      </c>
+      <c r="BH46">
+        <v>5</v>
+      </c>
+      <c r="BI46" t="s">
+        <v>90</v>
+      </c>
+      <c r="BJ46" t="s">
+        <v>90</v>
+      </c>
+      <c r="BK46">
+        <v>15</v>
+      </c>
+      <c r="BL46">
+        <v>17</v>
+      </c>
+      <c r="BM46">
+        <v>13</v>
+      </c>
+      <c r="BN46">
+        <v>16</v>
+      </c>
+      <c r="BO46">
+        <v>2</v>
+      </c>
+      <c r="BP46">
+        <v>3</v>
+      </c>
+      <c r="BQ46">
+        <v>24</v>
+      </c>
+      <c r="BR46">
+        <v>40</v>
+      </c>
+      <c r="BS46">
+        <v>0</v>
+      </c>
+      <c r="BT46">
+        <v>3</v>
+      </c>
+      <c r="BU46" t="s">
+        <v>90</v>
+      </c>
+      <c r="BV46" t="s">
+        <v>90</v>
+      </c>
+      <c r="BW46">
+        <v>62</v>
+      </c>
+      <c r="BX46">
+        <v>55</v>
+      </c>
+      <c r="BY46">
+        <v>37</v>
+      </c>
+      <c r="BZ46">
+        <v>29</v>
+      </c>
+      <c r="CA46">
+        <v>25</v>
+      </c>
+      <c r="CB46">
+        <v>26</v>
+      </c>
+      <c r="CC46">
+        <v>11</v>
+      </c>
+      <c r="CD46">
+        <v>1</v>
+      </c>
+      <c r="CE46" t="s">
+        <v>90</v>
+      </c>
+      <c r="CF46" t="s">
+        <v>90</v>
+      </c>
+      <c r="CG46">
+        <v>1</v>
+      </c>
+      <c r="CH46">
+        <v>1</v>
+      </c>
+      <c r="CI46">
+        <v>1</v>
+      </c>
+      <c r="CJ46">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Oct 17, 2026, 10:53 AM
</commit_message>
<xml_diff>
--- a/Bundesliga 26-27.xlsx
+++ b/Bundesliga 26-27.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kuba\Desktop\analityczka\26-27\Ekstraklasa 26-27\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{78DAC283-4B1C-4DF4-A956-DC2F011A8189}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{48492CC0-CE5C-4847-BC4B-2BB8E941C33F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{723BE2C8-720D-41E0-A496-B3B96A8488E1}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="582" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="593" uniqueCount="132">
   <si>
     <t>date</t>
   </si>
@@ -432,6 +432,9 @@
   </si>
   <si>
     <t>Sun 11 October, 17:30</t>
+  </si>
+  <si>
+    <t>Fri 16 October, 20:30</t>
   </si>
 </sst>
 </file>
@@ -849,7 +852,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9ED51FE2-0441-4690-9385-28E7CF18BF79}">
-  <dimension ref="B1:CJ46"/>
+  <dimension ref="B1:CJ47"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="17.7109375" customWidth="1"/>
@@ -1170,7 +1173,7 @@
         <v>59</v>
       </c>
       <c r="H2">
-        <f t="shared" ref="H2:H46" si="0">100-G2</f>
+        <f t="shared" ref="H2:H47" si="0">100-G2</f>
         <v>41</v>
       </c>
       <c r="I2">
@@ -13027,6 +13030,270 @@
         <v>1</v>
       </c>
       <c r="CJ46">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="2:88" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B47" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="C47" t="s">
+        <v>101</v>
+      </c>
+      <c r="D47" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="E47">
+        <v>1</v>
+      </c>
+      <c r="F47">
+        <v>0</v>
+      </c>
+      <c r="G47">
+        <v>56</v>
+      </c>
+      <c r="H47">
+        <f t="shared" si="0"/>
+        <v>44</v>
+      </c>
+      <c r="I47">
+        <v>1.8</v>
+      </c>
+      <c r="J47">
+        <v>0.8</v>
+      </c>
+      <c r="K47">
+        <v>15</v>
+      </c>
+      <c r="L47">
+        <v>9</v>
+      </c>
+      <c r="M47">
+        <v>7</v>
+      </c>
+      <c r="N47">
+        <v>3</v>
+      </c>
+      <c r="O47">
+        <v>3</v>
+      </c>
+      <c r="P47">
+        <v>2</v>
+      </c>
+      <c r="Q47">
+        <v>3</v>
+      </c>
+      <c r="R47">
+        <v>2</v>
+      </c>
+      <c r="S47">
+        <v>360</v>
+      </c>
+      <c r="T47">
+        <v>270</v>
+      </c>
+      <c r="U47">
+        <v>8</v>
+      </c>
+      <c r="V47">
+        <v>17</v>
+      </c>
+      <c r="W47">
+        <v>7</v>
+      </c>
+      <c r="X47">
+        <v>3</v>
+      </c>
+      <c r="Y47" t="s">
+        <v>90</v>
+      </c>
+      <c r="Z47" t="s">
+        <v>90</v>
+      </c>
+      <c r="AA47">
+        <v>4</v>
+      </c>
+      <c r="AB47">
+        <v>2</v>
+      </c>
+      <c r="AC47">
+        <v>4</v>
+      </c>
+      <c r="AD47">
+        <v>4</v>
+      </c>
+      <c r="AE47">
+        <v>0</v>
+      </c>
+      <c r="AF47">
+        <v>0</v>
+      </c>
+      <c r="AG47">
+        <v>11</v>
+      </c>
+      <c r="AH47">
+        <v>7</v>
+      </c>
+      <c r="AI47">
+        <v>4</v>
+      </c>
+      <c r="AJ47">
+        <v>2</v>
+      </c>
+      <c r="AK47">
+        <v>1.53</v>
+      </c>
+      <c r="AL47">
+        <v>0.5</v>
+      </c>
+      <c r="AM47">
+        <v>0.27</v>
+      </c>
+      <c r="AN47">
+        <v>0.3</v>
+      </c>
+      <c r="AO47">
+        <v>1.8</v>
+      </c>
+      <c r="AP47">
+        <v>0.8</v>
+      </c>
+      <c r="AQ47">
+        <v>1.78</v>
+      </c>
+      <c r="AR47">
+        <v>1.1399999999999999</v>
+      </c>
+      <c r="AS47">
+        <v>449</v>
+      </c>
+      <c r="AT47">
+        <v>360</v>
+      </c>
+      <c r="AU47">
+        <v>169</v>
+      </c>
+      <c r="AV47">
+        <v>133</v>
+      </c>
+      <c r="AW47">
+        <v>191</v>
+      </c>
+      <c r="AX47">
+        <v>137</v>
+      </c>
+      <c r="AY47">
+        <v>24</v>
+      </c>
+      <c r="AZ47">
+        <v>19</v>
+      </c>
+      <c r="BA47">
+        <v>5</v>
+      </c>
+      <c r="BB47">
+        <v>1</v>
+      </c>
+      <c r="BC47">
+        <v>31</v>
+      </c>
+      <c r="BD47">
+        <v>28</v>
+      </c>
+      <c r="BE47">
+        <v>28</v>
+      </c>
+      <c r="BF47">
+        <v>22</v>
+      </c>
+      <c r="BG47">
+        <v>1</v>
+      </c>
+      <c r="BH47">
+        <v>0</v>
+      </c>
+      <c r="BI47" t="s">
+        <v>90</v>
+      </c>
+      <c r="BJ47" t="s">
+        <v>90</v>
+      </c>
+      <c r="BK47">
+        <v>22</v>
+      </c>
+      <c r="BL47">
+        <v>29</v>
+      </c>
+      <c r="BM47">
+        <v>12</v>
+      </c>
+      <c r="BN47">
+        <v>12</v>
+      </c>
+      <c r="BO47">
+        <v>4</v>
+      </c>
+      <c r="BP47">
+        <v>4</v>
+      </c>
+      <c r="BQ47">
+        <v>27</v>
+      </c>
+      <c r="BR47">
+        <v>31</v>
+      </c>
+      <c r="BS47">
+        <v>3</v>
+      </c>
+      <c r="BT47">
+        <v>6</v>
+      </c>
+      <c r="BU47" t="s">
+        <v>90</v>
+      </c>
+      <c r="BV47" t="s">
+        <v>90</v>
+      </c>
+      <c r="BW47">
+        <v>70</v>
+      </c>
+      <c r="BX47">
+        <v>59</v>
+      </c>
+      <c r="BY47">
+        <v>46</v>
+      </c>
+      <c r="BZ47">
+        <v>38</v>
+      </c>
+      <c r="CA47">
+        <v>24</v>
+      </c>
+      <c r="CB47">
+        <v>21</v>
+      </c>
+      <c r="CC47">
+        <v>9</v>
+      </c>
+      <c r="CD47">
+        <v>3</v>
+      </c>
+      <c r="CE47" t="s">
+        <v>90</v>
+      </c>
+      <c r="CF47" t="s">
+        <v>90</v>
+      </c>
+      <c r="CG47">
+        <v>2</v>
+      </c>
+      <c r="CH47">
+        <v>2</v>
+      </c>
+      <c r="CI47">
+        <v>0</v>
+      </c>
+      <c r="CJ47">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Oct 17, 2026, 9:18 PM
</commit_message>
<xml_diff>
--- a/Bundesliga 26-27.xlsx
+++ b/Bundesliga 26-27.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kuba\Desktop\analityczka\26-27\Ekstraklasa 26-27\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kuba\Desktop\analityczka\26-27\Bundesliga 26-27\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{48492CC0-CE5C-4847-BC4B-2BB8E941C33F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A8EA9779-D062-4EAD-93A3-716C256C24CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{723BE2C8-720D-41E0-A496-B3B96A8488E1}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="593" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="560" uniqueCount="129">
   <si>
     <t>date</t>
   </si>
@@ -422,19 +422,10 @@
     <t>Fri 9 October, 20:30</t>
   </si>
   <si>
-    <t>Sat 10 October, 15:30</t>
-  </si>
-  <si>
-    <t>Sat 10 October, 18:30</t>
-  </si>
-  <si>
-    <t>Sun 11 October, 15:30</t>
-  </si>
-  <si>
-    <t>Sun 11 October, 17:30</t>
-  </si>
-  <si>
-    <t>Fri 16 October, 20:30</t>
+    <t>Sat 17 October, 15:30</t>
+  </si>
+  <si>
+    <t>Sat 17 October, 18:30</t>
   </si>
 </sst>
 </file>
@@ -852,7 +843,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9ED51FE2-0441-4690-9385-28E7CF18BF79}">
-  <dimension ref="B1:CJ47"/>
+  <dimension ref="B1:CJ44"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="17.7109375" customWidth="1"/>
@@ -1173,7 +1164,7 @@
         <v>59</v>
       </c>
       <c r="H2">
-        <f t="shared" ref="H2:H47" si="0">100-G2</f>
+        <f t="shared" ref="H2:H44" si="0">100-G2</f>
         <v>41</v>
       </c>
       <c r="I2">
@@ -10926,215 +10917,215 @@
         <v>127</v>
       </c>
       <c r="C39" t="s">
+        <v>92</v>
+      </c>
+      <c r="D39" t="s">
         <v>108</v>
       </c>
-      <c r="D39" s="2" t="s">
-        <v>87</v>
-      </c>
       <c r="E39">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F39">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G39">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="H39">
         <f t="shared" si="0"/>
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="I39">
-        <v>2.37</v>
+        <v>3.61</v>
       </c>
       <c r="J39">
-        <v>4.96</v>
+        <v>3.45</v>
       </c>
       <c r="K39">
+        <v>19</v>
+      </c>
+      <c r="L39">
+        <v>29</v>
+      </c>
+      <c r="M39">
+        <v>8</v>
+      </c>
+      <c r="N39">
+        <v>8</v>
+      </c>
+      <c r="O39">
+        <v>5</v>
+      </c>
+      <c r="P39">
+        <v>4</v>
+      </c>
+      <c r="Q39">
+        <v>2</v>
+      </c>
+      <c r="R39">
+        <v>2</v>
+      </c>
+      <c r="S39">
+        <v>252</v>
+      </c>
+      <c r="T39">
+        <v>379</v>
+      </c>
+      <c r="U39">
+        <v>16</v>
+      </c>
+      <c r="V39">
+        <v>14</v>
+      </c>
+      <c r="W39">
+        <v>4</v>
+      </c>
+      <c r="X39">
         <v>12</v>
       </c>
-      <c r="L39">
-        <v>30</v>
-      </c>
-      <c r="M39">
-        <v>5</v>
-      </c>
-      <c r="N39">
-        <v>10</v>
-      </c>
-      <c r="O39">
-        <v>3</v>
-      </c>
-      <c r="P39">
+      <c r="Y39" t="s">
+        <v>90</v>
+      </c>
+      <c r="Z39" t="s">
+        <v>90</v>
+      </c>
+      <c r="AA39">
+        <v>4</v>
+      </c>
+      <c r="AB39">
+        <v>9</v>
+      </c>
+      <c r="AC39">
         <v>7</v>
       </c>
-      <c r="Q39">
-        <v>1</v>
-      </c>
-      <c r="R39">
-        <v>5</v>
-      </c>
-      <c r="S39">
-        <v>217</v>
-      </c>
-      <c r="T39">
-        <v>582</v>
-      </c>
-      <c r="U39">
-        <v>10</v>
-      </c>
-      <c r="V39">
-        <v>6</v>
-      </c>
-      <c r="W39">
-        <v>5</v>
-      </c>
-      <c r="X39">
-        <v>9</v>
-      </c>
-      <c r="Y39" t="s">
-        <v>90</v>
-      </c>
-      <c r="Z39" t="s">
-        <v>90</v>
-      </c>
-      <c r="AA39">
-        <v>4</v>
-      </c>
-      <c r="AB39">
-        <v>11</v>
-      </c>
-      <c r="AC39">
-        <v>3</v>
-      </c>
       <c r="AD39">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="AE39">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AF39">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AG39">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="AH39">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="AI39">
         <v>2</v>
       </c>
       <c r="AJ39">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="AK39">
-        <v>1.74</v>
+        <v>1.57</v>
       </c>
       <c r="AL39">
-        <v>4.2300000000000004</v>
+        <v>1.06</v>
       </c>
       <c r="AM39">
-        <v>0.63</v>
+        <v>0.46</v>
       </c>
       <c r="AN39">
-        <v>0.73</v>
+        <v>0.82</v>
       </c>
       <c r="AO39">
-        <v>2.37</v>
+        <v>2.0299999999999998</v>
       </c>
       <c r="AP39">
-        <v>4.96</v>
+        <v>1.88</v>
       </c>
       <c r="AQ39">
-        <v>2</v>
+        <v>4.76</v>
       </c>
       <c r="AR39">
-        <v>4.29</v>
+        <v>2.2400000000000002</v>
       </c>
       <c r="AS39">
-        <v>286</v>
+        <v>326</v>
       </c>
       <c r="AT39">
-        <v>649</v>
+        <v>466</v>
       </c>
       <c r="AU39">
-        <v>124</v>
+        <v>156</v>
       </c>
       <c r="AV39">
-        <v>119</v>
+        <v>205</v>
       </c>
       <c r="AW39">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="AX39">
-        <v>463</v>
+        <v>174</v>
       </c>
       <c r="AY39">
         <v>24</v>
       </c>
       <c r="AZ39">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="BA39">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BB39">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="BC39">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="BD39">
+        <v>17</v>
+      </c>
+      <c r="BE39">
+        <v>34</v>
+      </c>
+      <c r="BF39">
+        <v>49</v>
+      </c>
+      <c r="BG39">
+        <v>3</v>
+      </c>
+      <c r="BH39">
+        <v>2</v>
+      </c>
+      <c r="BI39" t="s">
+        <v>90</v>
+      </c>
+      <c r="BJ39" t="s">
+        <v>90</v>
+      </c>
+      <c r="BK39">
         <v>22</v>
       </c>
-      <c r="BE39">
-        <v>23</v>
-      </c>
-      <c r="BF39">
-        <v>62</v>
-      </c>
-      <c r="BG39">
-        <v>1</v>
-      </c>
-      <c r="BH39">
-        <v>4</v>
-      </c>
-      <c r="BI39" t="s">
-        <v>90</v>
-      </c>
-      <c r="BJ39" t="s">
-        <v>90</v>
-      </c>
-      <c r="BK39">
-        <v>24</v>
-      </c>
       <c r="BL39">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="BM39">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="BN39">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="BO39">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="BP39">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="BQ39">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="BR39">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="BS39">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="BT39">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="BU39" t="s">
         <v>90</v>
@@ -11143,28 +11134,28 @@
         <v>90</v>
       </c>
       <c r="BW39">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="BX39">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="BY39">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="BZ39">
         <v>34</v>
       </c>
       <c r="CA39">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="CB39">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="CC39">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="CD39">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="CE39" t="s">
         <v>90</v>
@@ -11173,10 +11164,10 @@
         <v>90</v>
       </c>
       <c r="CG39">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="CH39">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="CI39">
         <v>0</v>
@@ -11189,247 +11180,247 @@
       <c r="B40" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="C40" t="s">
-        <v>95</v>
-      </c>
-      <c r="D40" s="4" t="s">
+      <c r="C40" s="4" t="s">
         <v>104</v>
       </c>
+      <c r="D40" t="s">
+        <v>88</v>
+      </c>
       <c r="E40">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F40">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G40">
-        <v>64</v>
+        <v>34</v>
       </c>
       <c r="H40">
         <f t="shared" si="0"/>
+        <v>66</v>
+      </c>
+      <c r="I40">
+        <v>1.42</v>
+      </c>
+      <c r="J40">
+        <v>1.69</v>
+      </c>
+      <c r="K40">
+        <v>14</v>
+      </c>
+      <c r="L40">
+        <v>24</v>
+      </c>
+      <c r="M40">
+        <v>3</v>
+      </c>
+      <c r="N40">
+        <v>5</v>
+      </c>
+      <c r="O40">
+        <v>3</v>
+      </c>
+      <c r="P40">
+        <v>6</v>
+      </c>
+      <c r="Q40">
+        <v>3</v>
+      </c>
+      <c r="R40">
+        <v>6</v>
+      </c>
+      <c r="S40">
+        <v>240</v>
+      </c>
+      <c r="T40">
+        <v>573</v>
+      </c>
+      <c r="U40">
+        <v>12</v>
+      </c>
+      <c r="V40">
+        <v>9</v>
+      </c>
+      <c r="W40">
+        <v>5</v>
+      </c>
+      <c r="X40">
+        <v>9</v>
+      </c>
+      <c r="Y40" t="s">
+        <v>90</v>
+      </c>
+      <c r="Z40" t="s">
+        <v>90</v>
+      </c>
+      <c r="AA40">
+        <v>9</v>
+      </c>
+      <c r="AB40">
+        <v>12</v>
+      </c>
+      <c r="AC40">
+        <v>2</v>
+      </c>
+      <c r="AD40">
+        <v>7</v>
+      </c>
+      <c r="AE40">
+        <v>1</v>
+      </c>
+      <c r="AF40">
+        <v>1</v>
+      </c>
+      <c r="AG40">
+        <v>8</v>
+      </c>
+      <c r="AH40">
+        <v>15</v>
+      </c>
+      <c r="AI40">
+        <v>6</v>
+      </c>
+      <c r="AJ40">
+        <v>9</v>
+      </c>
+      <c r="AK40">
+        <v>0.63</v>
+      </c>
+      <c r="AL40">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="AM40">
+        <v>0.8</v>
+      </c>
+      <c r="AN40">
+        <v>0.6</v>
+      </c>
+      <c r="AO40">
+        <v>1.42</v>
+      </c>
+      <c r="AP40">
+        <v>1.69</v>
+      </c>
+      <c r="AQ40">
+        <v>1.58</v>
+      </c>
+      <c r="AR40">
+        <v>1.41</v>
+      </c>
+      <c r="AS40">
+        <v>315</v>
+      </c>
+      <c r="AT40">
+        <v>625</v>
+      </c>
+      <c r="AU40">
+        <v>132</v>
+      </c>
+      <c r="AV40">
+        <v>198</v>
+      </c>
+      <c r="AW40">
+        <v>108</v>
+      </c>
+      <c r="AX40">
+        <v>375</v>
+      </c>
+      <c r="AY40">
+        <v>22</v>
+      </c>
+      <c r="AZ40">
+        <v>23</v>
+      </c>
+      <c r="BA40">
+        <v>6</v>
+      </c>
+      <c r="BB40">
+        <v>13</v>
+      </c>
+      <c r="BC40">
+        <v>13</v>
+      </c>
+      <c r="BD40">
+        <v>16</v>
+      </c>
+      <c r="BE40">
+        <v>21</v>
+      </c>
+      <c r="BF40">
+        <v>38</v>
+      </c>
+      <c r="BG40">
+        <v>0</v>
+      </c>
+      <c r="BH40">
+        <v>0</v>
+      </c>
+      <c r="BI40" t="s">
+        <v>90</v>
+      </c>
+      <c r="BJ40" t="s">
+        <v>90</v>
+      </c>
+      <c r="BK40">
+        <v>19</v>
+      </c>
+      <c r="BL40">
+        <v>10</v>
+      </c>
+      <c r="BM40">
+        <v>7</v>
+      </c>
+      <c r="BN40">
+        <v>7</v>
+      </c>
+      <c r="BO40">
+        <v>6</v>
+      </c>
+      <c r="BP40">
+        <v>1</v>
+      </c>
+      <c r="BQ40">
         <v>36</v>
       </c>
-      <c r="I40">
-        <v>0.93</v>
-      </c>
-      <c r="J40">
-        <v>1.28</v>
-      </c>
-      <c r="K40">
-        <v>17</v>
-      </c>
-      <c r="L40">
-        <v>15</v>
-      </c>
-      <c r="M40">
-        <v>4</v>
-      </c>
-      <c r="N40">
-        <v>4</v>
-      </c>
-      <c r="O40">
-        <v>3</v>
-      </c>
-      <c r="P40">
-        <v>3</v>
-      </c>
-      <c r="Q40">
-        <v>3</v>
-      </c>
-      <c r="R40">
-        <v>1</v>
-      </c>
-      <c r="S40">
-        <v>444</v>
-      </c>
-      <c r="T40">
-        <v>211</v>
-      </c>
-      <c r="U40">
-        <v>11</v>
-      </c>
-      <c r="V40">
-        <v>16</v>
-      </c>
-      <c r="W40">
+      <c r="BR40">
+        <v>32</v>
+      </c>
+      <c r="BS40">
+        <v>5</v>
+      </c>
+      <c r="BT40">
+        <v>2</v>
+      </c>
+      <c r="BU40" t="s">
+        <v>90</v>
+      </c>
+      <c r="BV40" t="s">
+        <v>90</v>
+      </c>
+      <c r="BW40">
+        <v>52</v>
+      </c>
+      <c r="BX40">
+        <v>52</v>
+      </c>
+      <c r="BY40">
+        <v>32</v>
+      </c>
+      <c r="BZ40">
+        <v>31</v>
+      </c>
+      <c r="CA40">
+        <v>20</v>
+      </c>
+      <c r="CB40">
+        <v>21</v>
+      </c>
+      <c r="CC40">
         <v>7</v>
       </c>
-      <c r="X40">
-        <v>3</v>
-      </c>
-      <c r="Y40" t="s">
-        <v>90</v>
-      </c>
-      <c r="Z40" t="s">
-        <v>90</v>
-      </c>
-      <c r="AA40">
-        <v>5</v>
-      </c>
-      <c r="AB40">
-        <v>7</v>
-      </c>
-      <c r="AC40">
-        <v>8</v>
-      </c>
-      <c r="AD40">
-        <v>4</v>
-      </c>
-      <c r="AE40">
-        <v>0</v>
-      </c>
-      <c r="AF40">
-        <v>1</v>
-      </c>
-      <c r="AG40">
+      <c r="CD40">
         <v>9</v>
       </c>
-      <c r="AH40">
-        <v>10</v>
-      </c>
-      <c r="AI40">
-        <v>8</v>
-      </c>
-      <c r="AJ40">
-        <v>5</v>
-      </c>
-      <c r="AK40">
-        <v>0.73</v>
-      </c>
-      <c r="AL40">
-        <v>0.62</v>
-      </c>
-      <c r="AM40">
-        <v>0.2</v>
-      </c>
-      <c r="AN40">
-        <v>0.66</v>
-      </c>
-      <c r="AO40">
-        <v>0.93</v>
-      </c>
-      <c r="AP40">
-        <v>1.28</v>
-      </c>
-      <c r="AQ40">
-        <v>0.68</v>
-      </c>
-      <c r="AR40">
-        <v>1.66</v>
-      </c>
-      <c r="AS40">
-        <v>545</v>
-      </c>
-      <c r="AT40">
-        <v>306</v>
-      </c>
-      <c r="AU40">
-        <v>188</v>
-      </c>
-      <c r="AV40">
-        <v>104</v>
-      </c>
-      <c r="AW40">
-        <v>256</v>
-      </c>
-      <c r="AX40">
-        <v>107</v>
-      </c>
-      <c r="AY40">
-        <v>20</v>
-      </c>
-      <c r="AZ40">
-        <v>25</v>
-      </c>
-      <c r="BA40">
-        <v>7</v>
-      </c>
-      <c r="BB40">
-        <v>5</v>
-      </c>
-      <c r="BC40">
-        <v>25</v>
-      </c>
-      <c r="BD40">
-        <v>17</v>
-      </c>
-      <c r="BE40">
-        <v>41</v>
-      </c>
-      <c r="BF40">
-        <v>19</v>
-      </c>
-      <c r="BG40">
-        <v>3</v>
-      </c>
-      <c r="BH40">
-        <v>1</v>
-      </c>
-      <c r="BI40" t="s">
-        <v>90</v>
-      </c>
-      <c r="BJ40" t="s">
-        <v>90</v>
-      </c>
-      <c r="BK40">
-        <v>13</v>
-      </c>
-      <c r="BL40">
-        <v>18</v>
-      </c>
-      <c r="BM40">
-        <v>15</v>
-      </c>
-      <c r="BN40">
-        <v>12</v>
-      </c>
-      <c r="BO40">
-        <v>4</v>
-      </c>
-      <c r="BP40">
-        <v>8</v>
-      </c>
-      <c r="BQ40">
-        <v>25</v>
-      </c>
-      <c r="BR40">
-        <v>40</v>
-      </c>
-      <c r="BS40">
-        <v>1</v>
-      </c>
-      <c r="BT40">
-        <v>3</v>
-      </c>
-      <c r="BU40" t="s">
-        <v>90</v>
-      </c>
-      <c r="BV40" t="s">
-        <v>90</v>
-      </c>
-      <c r="BW40">
-        <v>65</v>
-      </c>
-      <c r="BX40">
-        <v>49</v>
-      </c>
-      <c r="BY40">
-        <v>37</v>
-      </c>
-      <c r="BZ40">
-        <v>32</v>
-      </c>
-      <c r="CA40">
-        <v>28</v>
-      </c>
-      <c r="CB40">
-        <v>17</v>
-      </c>
-      <c r="CC40">
-        <v>10</v>
-      </c>
-      <c r="CD40">
-        <v>4</v>
-      </c>
       <c r="CE40" t="s">
         <v>90</v>
       </c>
@@ -11437,13 +11428,13 @@
         <v>90</v>
       </c>
       <c r="CG40">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CH40">
         <v>0</v>
       </c>
       <c r="CI40">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="CJ40">
         <v>0</v>
@@ -11454,16 +11445,16 @@
         <v>127</v>
       </c>
       <c r="C41" t="s">
+        <v>109</v>
+      </c>
+      <c r="D41" t="s">
         <v>96</v>
       </c>
-      <c r="D41" s="4" t="s">
-        <v>93</v>
-      </c>
       <c r="E41">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F41">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G41">
         <v>47</v>
@@ -11473,160 +11464,160 @@
         <v>53</v>
       </c>
       <c r="I41">
-        <v>2.87</v>
+        <v>0.43</v>
       </c>
       <c r="J41">
-        <v>1.69</v>
+        <v>1.94</v>
       </c>
       <c r="K41">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="L41">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="M41">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N41">
+        <v>6</v>
+      </c>
+      <c r="O41">
+        <v>1</v>
+      </c>
+      <c r="P41">
+        <v>4</v>
+      </c>
+      <c r="Q41">
+        <v>1</v>
+      </c>
+      <c r="R41">
+        <v>3</v>
+      </c>
+      <c r="S41">
+        <v>259</v>
+      </c>
+      <c r="T41">
+        <v>339</v>
+      </c>
+      <c r="U41">
+        <v>12</v>
+      </c>
+      <c r="V41">
+        <v>20</v>
+      </c>
+      <c r="W41">
+        <v>4</v>
+      </c>
+      <c r="X41">
+        <v>1</v>
+      </c>
+      <c r="Y41" t="s">
+        <v>90</v>
+      </c>
+      <c r="Z41" t="s">
+        <v>90</v>
+      </c>
+      <c r="AA41">
+        <v>2</v>
+      </c>
+      <c r="AB41">
+        <v>2</v>
+      </c>
+      <c r="AC41">
+        <v>4</v>
+      </c>
+      <c r="AD41">
+        <v>2</v>
+      </c>
+      <c r="AE41">
+        <v>0</v>
+      </c>
+      <c r="AF41">
+        <v>0</v>
+      </c>
+      <c r="AG41">
         <v>7</v>
       </c>
-      <c r="O41">
-        <v>2</v>
-      </c>
-      <c r="P41">
-        <v>4</v>
-      </c>
-      <c r="Q41">
-        <v>1</v>
-      </c>
-      <c r="R41">
-        <v>2</v>
-      </c>
-      <c r="S41">
-        <v>367</v>
-      </c>
-      <c r="T41">
-        <v>433</v>
-      </c>
-      <c r="U41">
-        <v>11</v>
-      </c>
-      <c r="V41">
-        <v>10</v>
-      </c>
-      <c r="W41">
-        <v>4</v>
-      </c>
-      <c r="X41">
-        <v>3</v>
-      </c>
-      <c r="Y41" t="s">
-        <v>90</v>
-      </c>
-      <c r="Z41" t="s">
-        <v>90</v>
-      </c>
-      <c r="AA41">
-        <v>11</v>
-      </c>
-      <c r="AB41">
-        <v>6</v>
-      </c>
-      <c r="AC41">
-        <v>7</v>
-      </c>
-      <c r="AD41">
-        <v>3</v>
-      </c>
-      <c r="AE41">
-        <v>0</v>
-      </c>
-      <c r="AF41">
-        <v>0</v>
-      </c>
-      <c r="AG41">
-        <v>17</v>
-      </c>
       <c r="AH41">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AI41">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="AJ41">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AK41">
-        <v>1.24</v>
+        <v>0.05</v>
       </c>
       <c r="AL41">
-        <v>1.54</v>
+        <v>1.92</v>
       </c>
       <c r="AM41">
-        <v>1.63</v>
+        <v>0.38</v>
       </c>
       <c r="AN41">
-        <v>0.15</v>
+        <v>0.02</v>
       </c>
       <c r="AO41">
-        <v>2.87</v>
+        <v>0.43</v>
       </c>
       <c r="AP41">
-        <v>1.69</v>
+        <v>1.94</v>
       </c>
       <c r="AQ41">
-        <v>1.39</v>
+        <v>0.4</v>
       </c>
       <c r="AR41">
-        <v>2.5099999999999998</v>
+        <v>2.98</v>
       </c>
       <c r="AS41">
-        <v>442</v>
+        <v>392</v>
       </c>
       <c r="AT41">
-        <v>508</v>
+        <v>462</v>
       </c>
       <c r="AU41">
-        <v>176</v>
+        <v>127</v>
       </c>
       <c r="AV41">
-        <v>215</v>
+        <v>197</v>
       </c>
       <c r="AW41">
-        <v>191</v>
+        <v>132</v>
       </c>
       <c r="AX41">
-        <v>218</v>
+        <v>142</v>
       </c>
       <c r="AY41">
         <v>16</v>
       </c>
       <c r="AZ41">
-        <v>22</v>
+        <v>35</v>
       </c>
       <c r="BA41">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="BB41">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BC41">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="BD41">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="BE41">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="BF41">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="BG41">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="BH41">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="BI41" t="s">
         <v>90</v>
@@ -11635,34 +11626,34 @@
         <v>90</v>
       </c>
       <c r="BK41">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="BL41">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="BM41">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="BN41">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="BO41">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="BP41">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="BQ41">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="BR41">
-        <v>20</v>
+        <v>51</v>
       </c>
       <c r="BS41">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="BT41">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BU41" t="s">
         <v>90</v>
@@ -11671,28 +11662,28 @@
         <v>90</v>
       </c>
       <c r="BW41">
-        <v>43</v>
+        <v>66</v>
       </c>
       <c r="BX41">
-        <v>37</v>
+        <v>60</v>
       </c>
       <c r="BY41">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="BZ41">
         <v>31</v>
       </c>
       <c r="CA41">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="CB41">
-        <v>6</v>
+        <v>29</v>
       </c>
       <c r="CC41">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="CD41">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="CE41" t="s">
         <v>90</v>
@@ -11701,10 +11692,10 @@
         <v>90</v>
       </c>
       <c r="CG41">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="CH41">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="CI41">
         <v>0</v>
@@ -11713,251 +11704,251 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="2:88" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:88" ht="30" x14ac:dyDescent="0.25">
       <c r="B42" s="3" t="s">
         <v>127</v>
       </c>
       <c r="C42" t="s">
-        <v>97</v>
-      </c>
-      <c r="D42" t="s">
-        <v>88</v>
+        <v>100</v>
+      </c>
+      <c r="D42" s="4" t="s">
+        <v>103</v>
       </c>
       <c r="E42">
         <v>0</v>
       </c>
       <c r="F42">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G42">
-        <v>52</v>
+        <v>37</v>
       </c>
       <c r="H42">
         <f t="shared" si="0"/>
-        <v>48</v>
+        <v>63</v>
       </c>
       <c r="I42">
-        <v>1.96</v>
+        <v>0.82</v>
       </c>
       <c r="J42">
-        <v>2.4700000000000002</v>
+        <v>1.36</v>
       </c>
       <c r="K42">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="L42">
+        <v>12</v>
+      </c>
+      <c r="M42">
+        <v>0</v>
+      </c>
+      <c r="N42">
+        <v>2</v>
+      </c>
+      <c r="O42">
+        <v>1</v>
+      </c>
+      <c r="P42">
+        <v>1</v>
+      </c>
+      <c r="Q42">
+        <v>1</v>
+      </c>
+      <c r="R42">
+        <v>1</v>
+      </c>
+      <c r="S42">
+        <v>246</v>
+      </c>
+      <c r="T42">
+        <v>500</v>
+      </c>
+      <c r="U42">
+        <v>13</v>
+      </c>
+      <c r="V42">
+        <v>12</v>
+      </c>
+      <c r="W42">
+        <v>5</v>
+      </c>
+      <c r="X42">
+        <v>5</v>
+      </c>
+      <c r="Y42" t="s">
+        <v>90</v>
+      </c>
+      <c r="Z42" t="s">
+        <v>90</v>
+      </c>
+      <c r="AA42">
+        <v>8</v>
+      </c>
+      <c r="AB42">
+        <v>8</v>
+      </c>
+      <c r="AC42">
+        <v>3</v>
+      </c>
+      <c r="AD42">
+        <v>2</v>
+      </c>
+      <c r="AE42">
+        <v>0</v>
+      </c>
+      <c r="AF42">
+        <v>0</v>
+      </c>
+      <c r="AG42">
+        <v>5</v>
+      </c>
+      <c r="AH42">
+        <v>10</v>
+      </c>
+      <c r="AI42">
+        <v>6</v>
+      </c>
+      <c r="AJ42">
+        <v>2</v>
+      </c>
+      <c r="AK42">
+        <v>0.18</v>
+      </c>
+      <c r="AL42">
+        <v>1.17</v>
+      </c>
+      <c r="AM42">
+        <v>0.64</v>
+      </c>
+      <c r="AN42">
+        <v>0.19</v>
+      </c>
+      <c r="AO42">
+        <v>0.82</v>
+      </c>
+      <c r="AP42">
+        <v>1.36</v>
+      </c>
+      <c r="AQ42">
+        <v>0</v>
+      </c>
+      <c r="AR42">
+        <v>0.09</v>
+      </c>
+      <c r="AS42">
+        <v>340</v>
+      </c>
+      <c r="AT42">
+        <v>570</v>
+      </c>
+      <c r="AU42">
+        <v>118</v>
+      </c>
+      <c r="AV42">
+        <v>261</v>
+      </c>
+      <c r="AW42">
+        <v>129</v>
+      </c>
+      <c r="AX42">
+        <v>239</v>
+      </c>
+      <c r="AY42">
+        <v>26</v>
+      </c>
+      <c r="AZ42">
+        <v>21</v>
+      </c>
+      <c r="BA42">
+        <v>4</v>
+      </c>
+      <c r="BB42">
+        <v>8</v>
+      </c>
+      <c r="BC42">
+        <v>21</v>
+      </c>
+      <c r="BD42">
+        <v>16</v>
+      </c>
+      <c r="BE42">
+        <v>12</v>
+      </c>
+      <c r="BF42">
+        <v>31</v>
+      </c>
+      <c r="BG42">
+        <v>0</v>
+      </c>
+      <c r="BH42">
+        <v>1</v>
+      </c>
+      <c r="BI42" t="s">
+        <v>90</v>
+      </c>
+      <c r="BJ42" t="s">
+        <v>90</v>
+      </c>
+      <c r="BK42">
         <v>18</v>
       </c>
-      <c r="M42">
-        <v>6</v>
-      </c>
-      <c r="N42">
+      <c r="BL42">
+        <v>14</v>
+      </c>
+      <c r="BM42">
+        <v>9</v>
+      </c>
+      <c r="BN42">
+        <v>7</v>
+      </c>
+      <c r="BO42">
+        <v>1</v>
+      </c>
+      <c r="BP42">
+        <v>3</v>
+      </c>
+      <c r="BQ42">
+        <v>29</v>
+      </c>
+      <c r="BR42">
+        <v>40</v>
+      </c>
+      <c r="BS42">
+        <v>2</v>
+      </c>
+      <c r="BT42">
+        <v>0</v>
+      </c>
+      <c r="BU42" t="s">
+        <v>90</v>
+      </c>
+      <c r="BV42" t="s">
+        <v>90</v>
+      </c>
+      <c r="BW42">
+        <v>53</v>
+      </c>
+      <c r="BX42">
+        <v>52</v>
+      </c>
+      <c r="BY42">
+        <v>37</v>
+      </c>
+      <c r="BZ42">
+        <v>34</v>
+      </c>
+      <c r="CA42">
+        <v>16</v>
+      </c>
+      <c r="CB42">
+        <v>18</v>
+      </c>
+      <c r="CC42">
+        <v>7</v>
+      </c>
+      <c r="CD42">
         <v>8</v>
       </c>
-      <c r="O42">
-        <v>4</v>
-      </c>
-      <c r="P42">
-        <v>6</v>
-      </c>
-      <c r="Q42">
-        <v>4</v>
-      </c>
-      <c r="R42">
-        <v>5</v>
-      </c>
-      <c r="S42">
-        <v>400</v>
-      </c>
-      <c r="T42">
-        <v>358</v>
-      </c>
-      <c r="U42">
-        <v>10</v>
-      </c>
-      <c r="V42">
-        <v>11</v>
-      </c>
-      <c r="W42">
-        <v>7</v>
-      </c>
-      <c r="X42">
-        <v>5</v>
-      </c>
-      <c r="Y42" t="s">
-        <v>90</v>
-      </c>
-      <c r="Z42" t="s">
-        <v>90</v>
-      </c>
-      <c r="AA42">
-        <v>10</v>
-      </c>
-      <c r="AB42">
-        <v>5</v>
-      </c>
-      <c r="AC42">
-        <v>8</v>
-      </c>
-      <c r="AD42">
-        <v>5</v>
-      </c>
-      <c r="AE42">
-        <v>0</v>
-      </c>
-      <c r="AF42">
-        <v>1</v>
-      </c>
-      <c r="AG42">
-        <v>16</v>
-      </c>
-      <c r="AH42">
-        <v>16</v>
-      </c>
-      <c r="AI42">
-        <v>8</v>
-      </c>
-      <c r="AJ42">
-        <v>2</v>
-      </c>
-      <c r="AK42">
-        <v>1.51</v>
-      </c>
-      <c r="AL42">
-        <v>2.02</v>
-      </c>
-      <c r="AM42">
-        <v>0.45</v>
-      </c>
-      <c r="AN42">
-        <v>0.46</v>
-      </c>
-      <c r="AO42">
-        <v>1.96</v>
-      </c>
-      <c r="AP42">
-        <v>2.4700000000000002</v>
-      </c>
-      <c r="AQ42">
-        <v>0.4</v>
-      </c>
-      <c r="AR42">
-        <v>1.85</v>
-      </c>
-      <c r="AS42">
-        <v>489</v>
-      </c>
-      <c r="AT42">
-        <v>458</v>
-      </c>
-      <c r="AU42">
-        <v>209</v>
-      </c>
-      <c r="AV42">
-        <v>217</v>
-      </c>
-      <c r="AW42">
-        <v>191</v>
-      </c>
-      <c r="AX42">
-        <v>141</v>
-      </c>
-      <c r="AY42">
-        <v>22</v>
-      </c>
-      <c r="AZ42">
-        <v>28</v>
-      </c>
-      <c r="BA42">
-        <v>8</v>
-      </c>
-      <c r="BB42">
-        <v>4</v>
-      </c>
-      <c r="BC42">
-        <v>19</v>
-      </c>
-      <c r="BD42">
-        <v>15</v>
-      </c>
-      <c r="BE42">
-        <v>36</v>
-      </c>
-      <c r="BF42">
-        <v>34</v>
-      </c>
-      <c r="BG42">
-        <v>1</v>
-      </c>
-      <c r="BH42">
-        <v>1</v>
-      </c>
-      <c r="BI42" t="s">
-        <v>90</v>
-      </c>
-      <c r="BJ42" t="s">
-        <v>90</v>
-      </c>
-      <c r="BK42">
-        <v>23</v>
-      </c>
-      <c r="BL42">
-        <v>21</v>
-      </c>
-      <c r="BM42">
-        <v>15</v>
-      </c>
-      <c r="BN42">
-        <v>10</v>
-      </c>
-      <c r="BO42">
-        <v>6</v>
-      </c>
-      <c r="BP42">
-        <v>10</v>
-      </c>
-      <c r="BQ42">
-        <v>15</v>
-      </c>
-      <c r="BR42">
-        <v>41</v>
-      </c>
-      <c r="BS42">
-        <v>5</v>
-      </c>
-      <c r="BT42">
-        <v>4</v>
-      </c>
-      <c r="BU42" t="s">
-        <v>90</v>
-      </c>
-      <c r="BV42" t="s">
-        <v>90</v>
-      </c>
-      <c r="BW42">
-        <v>64</v>
-      </c>
-      <c r="BX42">
-        <v>62</v>
-      </c>
-      <c r="BY42">
-        <v>45</v>
-      </c>
-      <c r="BZ42">
-        <v>38</v>
-      </c>
-      <c r="CA42">
-        <v>19</v>
-      </c>
-      <c r="CB42">
-        <v>24</v>
-      </c>
-      <c r="CC42">
-        <v>11</v>
-      </c>
-      <c r="CD42">
-        <v>7</v>
-      </c>
       <c r="CE42" t="s">
         <v>90</v>
       </c>
@@ -11965,10 +11956,10 @@
         <v>90</v>
       </c>
       <c r="CG42">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="CH42">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="CI42">
         <v>0</v>
@@ -11982,68 +11973,68 @@
         <v>127</v>
       </c>
       <c r="C43" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="D43" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E43">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F43">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G43">
-        <v>43</v>
+        <v>61</v>
       </c>
       <c r="H43">
         <f t="shared" si="0"/>
-        <v>57</v>
+        <v>39</v>
       </c>
       <c r="I43">
-        <v>1.1299999999999999</v>
+        <v>3.21</v>
       </c>
       <c r="J43">
-        <v>0.24</v>
+        <v>1.1499999999999999</v>
       </c>
       <c r="K43">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="L43">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="M43">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="N43">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O43">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="P43">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q43">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="R43">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S43">
-        <v>252</v>
+        <v>536</v>
       </c>
       <c r="T43">
-        <v>368</v>
+        <v>317</v>
       </c>
       <c r="U43">
+        <v>11</v>
+      </c>
+      <c r="V43">
         <v>14</v>
       </c>
-      <c r="V43">
-        <v>9</v>
-      </c>
       <c r="W43">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="X43">
         <v>3</v>
@@ -12055,106 +12046,106 @@
         <v>90</v>
       </c>
       <c r="AA43">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="AB43">
         <v>5</v>
       </c>
       <c r="AC43">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="AD43">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AE43">
         <v>0</v>
       </c>
       <c r="AF43">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AG43">
         <v>13</v>
       </c>
       <c r="AH43">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="AI43">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AJ43">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AK43">
-        <v>0.73</v>
+        <v>2.34</v>
       </c>
       <c r="AL43">
-        <v>0.08</v>
+        <v>0.6</v>
       </c>
       <c r="AM43">
-        <v>0.41</v>
+        <v>0.09</v>
       </c>
       <c r="AN43">
-        <v>0.16</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="AO43">
-        <v>1.1299999999999999</v>
+        <v>2.4300000000000002</v>
       </c>
       <c r="AP43">
-        <v>0.24</v>
+        <v>1.1499999999999999</v>
       </c>
       <c r="AQ43">
-        <v>1.0900000000000001</v>
+        <v>3.56</v>
       </c>
       <c r="AR43">
-        <v>0.15</v>
+        <v>1.29</v>
       </c>
       <c r="AS43">
-        <v>326</v>
+        <v>628</v>
       </c>
       <c r="AT43">
-        <v>452</v>
+        <v>399</v>
       </c>
       <c r="AU43">
-        <v>142</v>
+        <v>292</v>
       </c>
       <c r="AV43">
-        <v>232</v>
+        <v>177</v>
       </c>
       <c r="AW43">
-        <v>110</v>
+        <v>244</v>
       </c>
       <c r="AX43">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="AY43">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="AZ43">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="BA43">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="BB43">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="BC43">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="BD43">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="BE43">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="BF43">
         <v>22</v>
       </c>
       <c r="BG43">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="BH43">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="BI43" t="s">
         <v>90</v>
@@ -12163,65 +12154,65 @@
         <v>90</v>
       </c>
       <c r="BK43">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="BL43">
+        <v>26</v>
+      </c>
+      <c r="BM43">
+        <v>6</v>
+      </c>
+      <c r="BN43">
         <v>12</v>
       </c>
-      <c r="BM43">
-        <v>17</v>
-      </c>
-      <c r="BN43">
-        <v>7</v>
-      </c>
       <c r="BO43">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="BP43">
+        <v>2</v>
+      </c>
+      <c r="BQ43">
+        <v>26</v>
+      </c>
+      <c r="BR43">
+        <v>38</v>
+      </c>
+      <c r="BS43">
+        <v>2</v>
+      </c>
+      <c r="BT43">
+        <v>9</v>
+      </c>
+      <c r="BU43" t="s">
+        <v>90</v>
+      </c>
+      <c r="BV43" t="s">
+        <v>90</v>
+      </c>
+      <c r="BW43">
+        <v>62</v>
+      </c>
+      <c r="BX43">
+        <v>63</v>
+      </c>
+      <c r="BY43">
+        <v>41</v>
+      </c>
+      <c r="BZ43">
+        <v>43</v>
+      </c>
+      <c r="CA43">
+        <v>21</v>
+      </c>
+      <c r="CB43">
+        <v>20</v>
+      </c>
+      <c r="CC43">
+        <v>10</v>
+      </c>
+      <c r="CD43">
         <v>6</v>
       </c>
-      <c r="BQ43">
-        <v>29</v>
-      </c>
-      <c r="BR43">
-        <v>28</v>
-      </c>
-      <c r="BS43">
-        <v>2</v>
-      </c>
-      <c r="BT43">
-        <v>5</v>
-      </c>
-      <c r="BU43" t="s">
-        <v>90</v>
-      </c>
-      <c r="BV43" t="s">
-        <v>90</v>
-      </c>
-      <c r="BW43">
-        <v>49</v>
-      </c>
-      <c r="BX43">
-        <v>51</v>
-      </c>
-      <c r="BY43">
-        <v>31</v>
-      </c>
-      <c r="BZ43">
-        <v>30</v>
-      </c>
-      <c r="CA43">
-        <v>18</v>
-      </c>
-      <c r="CB43">
-        <v>21</v>
-      </c>
-      <c r="CC43">
-        <v>7</v>
-      </c>
-      <c r="CD43">
-        <v>5</v>
-      </c>
       <c r="CE43" t="s">
         <v>90</v>
       </c>
@@ -12229,7 +12220,7 @@
         <v>90</v>
       </c>
       <c r="CG43">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CH43">
         <v>1</v>
@@ -12245,72 +12236,72 @@
       <c r="B44" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="C44" t="s">
+      <c r="C44" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D44" t="s">
         <v>98</v>
-      </c>
-      <c r="D44" t="s">
-        <v>101</v>
       </c>
       <c r="E44">
         <v>6</v>
       </c>
       <c r="F44">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G44">
-        <v>47</v>
+        <v>62</v>
       </c>
       <c r="H44">
         <f t="shared" si="0"/>
-        <v>53</v>
+        <v>38</v>
       </c>
       <c r="I44">
-        <v>4.03</v>
+        <v>3.76</v>
       </c>
       <c r="J44">
-        <v>1.46</v>
+        <v>0.84</v>
       </c>
       <c r="K44">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="L44">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="M44">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="N44">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="O44">
         <v>8</v>
       </c>
       <c r="P44">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="Q44">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="R44">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="S44">
-        <v>376</v>
+        <v>601</v>
       </c>
       <c r="T44">
-        <v>423</v>
+        <v>337</v>
       </c>
       <c r="U44">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="V44">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="W44">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="X44">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="Y44" t="s">
         <v>90</v>
@@ -12319,143 +12310,143 @@
         <v>90</v>
       </c>
       <c r="AA44">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AB44">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AC44">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="AD44">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AE44">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AF44">
         <v>0</v>
       </c>
       <c r="AG44">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="AH44">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="AI44">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="AJ44">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AK44">
-        <v>3.05</v>
+        <v>3.31</v>
       </c>
       <c r="AL44">
-        <v>1.17</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="AM44">
-        <v>0.97</v>
+        <v>0.45</v>
       </c>
       <c r="AN44">
         <v>0.28000000000000003</v>
       </c>
       <c r="AO44">
-        <v>4.03</v>
+        <v>3.76</v>
       </c>
       <c r="AP44">
-        <v>1.46</v>
+        <v>0.84</v>
       </c>
       <c r="AQ44">
-        <v>4.9800000000000004</v>
+        <v>4.34</v>
       </c>
       <c r="AR44">
-        <v>2.33</v>
+        <v>0.73</v>
       </c>
       <c r="AS44">
-        <v>434</v>
+        <v>666</v>
       </c>
       <c r="AT44">
-        <v>486</v>
+        <v>412</v>
       </c>
       <c r="AU44">
-        <v>256</v>
+        <v>272</v>
       </c>
       <c r="AV44">
-        <v>218</v>
+        <v>224</v>
       </c>
       <c r="AW44">
-        <v>120</v>
+        <v>329</v>
       </c>
       <c r="AX44">
-        <v>205</v>
+        <v>113</v>
       </c>
       <c r="AY44">
+        <v>28</v>
+      </c>
+      <c r="AZ44">
+        <v>12</v>
+      </c>
+      <c r="BA44">
+        <v>3</v>
+      </c>
+      <c r="BB44">
+        <v>2</v>
+      </c>
+      <c r="BC44">
+        <v>15</v>
+      </c>
+      <c r="BD44">
+        <v>13</v>
+      </c>
+      <c r="BE44">
+        <v>48</v>
+      </c>
+      <c r="BF44">
+        <v>23</v>
+      </c>
+      <c r="BG44">
+        <v>4</v>
+      </c>
+      <c r="BH44">
+        <v>2</v>
+      </c>
+      <c r="BI44" t="s">
+        <v>90</v>
+      </c>
+      <c r="BJ44" t="s">
+        <v>90</v>
+      </c>
+      <c r="BK44">
+        <v>13</v>
+      </c>
+      <c r="BL44">
+        <v>19</v>
+      </c>
+      <c r="BM44">
+        <v>12</v>
+      </c>
+      <c r="BN44">
+        <v>13</v>
+      </c>
+      <c r="BO44">
+        <v>5</v>
+      </c>
+      <c r="BP44">
+        <v>8</v>
+      </c>
+      <c r="BQ44">
+        <v>8</v>
+      </c>
+      <c r="BR44">
         <v>25</v>
       </c>
-      <c r="AZ44">
-        <v>23</v>
-      </c>
-      <c r="BA44">
-        <v>5</v>
-      </c>
-      <c r="BB44">
-        <v>6</v>
-      </c>
-      <c r="BC44">
-        <v>17</v>
-      </c>
-      <c r="BD44">
-        <v>15</v>
-      </c>
-      <c r="BE44">
-        <v>37</v>
-      </c>
-      <c r="BF44">
-        <v>32</v>
-      </c>
-      <c r="BG44">
-        <v>1</v>
-      </c>
-      <c r="BH44">
-        <v>2</v>
-      </c>
-      <c r="BI44" t="s">
-        <v>90</v>
-      </c>
-      <c r="BJ44" t="s">
-        <v>90</v>
-      </c>
-      <c r="BK44">
-        <v>24</v>
-      </c>
-      <c r="BL44">
-        <v>20</v>
-      </c>
-      <c r="BM44">
-        <v>8</v>
-      </c>
-      <c r="BN44">
+      <c r="BS44">
+        <v>3</v>
+      </c>
+      <c r="BT44">
         <v>11</v>
       </c>
-      <c r="BO44">
-        <v>4</v>
-      </c>
-      <c r="BP44">
-        <v>4</v>
-      </c>
-      <c r="BQ44">
-        <v>26</v>
-      </c>
-      <c r="BR44">
-        <v>17</v>
-      </c>
-      <c r="BS44">
-        <v>9</v>
-      </c>
-      <c r="BT44">
-        <v>4</v>
-      </c>
       <c r="BU44" t="s">
         <v>90</v>
       </c>
@@ -12463,29 +12454,29 @@
         <v>90</v>
       </c>
       <c r="BW44">
-        <v>57</v>
+        <v>25</v>
       </c>
       <c r="BX44">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="BY44">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="BZ44">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="CA44">
+        <v>3</v>
+      </c>
+      <c r="CB44">
+        <v>5</v>
+      </c>
+      <c r="CC44">
+        <v>3</v>
+      </c>
+      <c r="CD44">
         <v>11</v>
       </c>
-      <c r="CB44">
-        <v>10</v>
-      </c>
-      <c r="CC44">
-        <v>10</v>
-      </c>
-      <c r="CD44">
-        <v>7</v>
-      </c>
       <c r="CE44" t="s">
         <v>90</v>
       </c>
@@ -12496,804 +12487,12 @@
         <v>1</v>
       </c>
       <c r="CH44">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="CI44">
         <v>0</v>
       </c>
       <c r="CJ44">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45" spans="2:88" ht="30" x14ac:dyDescent="0.25">
-      <c r="B45" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="C45" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="D45" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="E45">
-        <v>2</v>
-      </c>
-      <c r="F45">
-        <v>1</v>
-      </c>
-      <c r="G45">
-        <v>48</v>
-      </c>
-      <c r="H45">
-        <f t="shared" si="0"/>
-        <v>52</v>
-      </c>
-      <c r="I45">
-        <v>1.32</v>
-      </c>
-      <c r="J45">
-        <v>1.17</v>
-      </c>
-      <c r="K45">
-        <v>19</v>
-      </c>
-      <c r="L45">
-        <v>16</v>
-      </c>
-      <c r="M45">
-        <v>7</v>
-      </c>
-      <c r="N45">
-        <v>7</v>
-      </c>
-      <c r="O45">
-        <v>2</v>
-      </c>
-      <c r="P45">
-        <v>2</v>
-      </c>
-      <c r="Q45">
-        <v>2</v>
-      </c>
-      <c r="R45">
-        <v>1</v>
-      </c>
-      <c r="S45">
-        <v>312</v>
-      </c>
-      <c r="T45">
-        <v>339</v>
-      </c>
-      <c r="U45">
-        <v>8</v>
-      </c>
-      <c r="V45">
-        <v>17</v>
-      </c>
-      <c r="W45">
-        <v>6</v>
-      </c>
-      <c r="X45">
-        <v>6</v>
-      </c>
-      <c r="Y45" t="s">
-        <v>90</v>
-      </c>
-      <c r="Z45" t="s">
-        <v>90</v>
-      </c>
-      <c r="AA45">
-        <v>10</v>
-      </c>
-      <c r="AB45">
-        <v>4</v>
-      </c>
-      <c r="AC45">
-        <v>2</v>
-      </c>
-      <c r="AD45">
-        <v>5</v>
-      </c>
-      <c r="AE45">
-        <v>0</v>
-      </c>
-      <c r="AF45">
-        <v>0</v>
-      </c>
-      <c r="AG45">
-        <v>13</v>
-      </c>
-      <c r="AH45">
-        <v>7</v>
-      </c>
-      <c r="AI45">
-        <v>6</v>
-      </c>
-      <c r="AJ45">
-        <v>9</v>
-      </c>
-      <c r="AK45">
-        <v>0.9</v>
-      </c>
-      <c r="AL45">
-        <v>0.96</v>
-      </c>
-      <c r="AM45">
-        <v>0.42</v>
-      </c>
-      <c r="AN45">
-        <v>0.21</v>
-      </c>
-      <c r="AO45">
-        <v>1.32</v>
-      </c>
-      <c r="AP45">
-        <v>1.17</v>
-      </c>
-      <c r="AQ45">
-        <v>1.39</v>
-      </c>
-      <c r="AR45">
-        <v>1.77</v>
-      </c>
-      <c r="AS45">
-        <v>391</v>
-      </c>
-      <c r="AT45">
-        <v>422</v>
-      </c>
-      <c r="AU45">
-        <v>184</v>
-      </c>
-      <c r="AV45">
-        <v>159</v>
-      </c>
-      <c r="AW45">
-        <v>128</v>
-      </c>
-      <c r="AX45">
-        <v>180</v>
-      </c>
-      <c r="AY45">
-        <v>22</v>
-      </c>
-      <c r="AZ45">
-        <v>22</v>
-      </c>
-      <c r="BA45">
-        <v>5</v>
-      </c>
-      <c r="BB45">
-        <v>3</v>
-      </c>
-      <c r="BC45">
-        <v>14</v>
-      </c>
-      <c r="BD45">
-        <v>20</v>
-      </c>
-      <c r="BE45">
-        <v>28</v>
-      </c>
-      <c r="BF45">
-        <v>26</v>
-      </c>
-      <c r="BG45">
-        <v>1</v>
-      </c>
-      <c r="BH45">
-        <v>1</v>
-      </c>
-      <c r="BI45" t="s">
-        <v>90</v>
-      </c>
-      <c r="BJ45" t="s">
-        <v>90</v>
-      </c>
-      <c r="BK45">
-        <v>22</v>
-      </c>
-      <c r="BL45">
-        <v>9</v>
-      </c>
-      <c r="BM45">
-        <v>12</v>
-      </c>
-      <c r="BN45">
-        <v>4</v>
-      </c>
-      <c r="BO45">
-        <v>5</v>
-      </c>
-      <c r="BP45">
-        <v>2</v>
-      </c>
-      <c r="BQ45">
-        <v>34</v>
-      </c>
-      <c r="BR45">
-        <v>23</v>
-      </c>
-      <c r="BS45">
-        <v>6</v>
-      </c>
-      <c r="BT45">
-        <v>5</v>
-      </c>
-      <c r="BU45" t="s">
-        <v>90</v>
-      </c>
-      <c r="BV45" t="s">
-        <v>90</v>
-      </c>
-      <c r="BW45">
-        <v>65</v>
-      </c>
-      <c r="BX45">
-        <v>41</v>
-      </c>
-      <c r="BY45">
-        <v>48</v>
-      </c>
-      <c r="BZ45">
-        <v>23</v>
-      </c>
-      <c r="CA45">
-        <v>17</v>
-      </c>
-      <c r="CB45">
-        <v>18</v>
-      </c>
-      <c r="CC45">
-        <v>9</v>
-      </c>
-      <c r="CD45">
-        <v>6</v>
-      </c>
-      <c r="CE45" t="s">
-        <v>90</v>
-      </c>
-      <c r="CF45" t="s">
-        <v>90</v>
-      </c>
-      <c r="CG45">
-        <v>1</v>
-      </c>
-      <c r="CH45">
-        <v>3</v>
-      </c>
-      <c r="CI45">
-        <v>0</v>
-      </c>
-      <c r="CJ45">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46" spans="2:88" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="B46" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="C46" t="s">
-        <v>106</v>
-      </c>
-      <c r="D46" t="s">
-        <v>109</v>
-      </c>
-      <c r="E46">
-        <v>2</v>
-      </c>
-      <c r="F46">
-        <v>1</v>
-      </c>
-      <c r="G46">
-        <v>51</v>
-      </c>
-      <c r="H46">
-        <f t="shared" si="0"/>
-        <v>49</v>
-      </c>
-      <c r="I46">
-        <v>1.1499999999999999</v>
-      </c>
-      <c r="J46">
-        <v>0.32</v>
-      </c>
-      <c r="K46">
-        <v>10</v>
-      </c>
-      <c r="L46">
-        <v>5</v>
-      </c>
-      <c r="M46">
-        <v>4</v>
-      </c>
-      <c r="N46">
-        <v>1</v>
-      </c>
-      <c r="O46">
-        <v>5</v>
-      </c>
-      <c r="P46">
-        <v>0</v>
-      </c>
-      <c r="Q46">
-        <v>3</v>
-      </c>
-      <c r="R46">
-        <v>0</v>
-      </c>
-      <c r="S46">
-        <v>334</v>
-      </c>
-      <c r="T46">
-        <v>328</v>
-      </c>
-      <c r="U46">
-        <v>11</v>
-      </c>
-      <c r="V46">
-        <v>13</v>
-      </c>
-      <c r="W46">
-        <v>7</v>
-      </c>
-      <c r="X46">
-        <v>2</v>
-      </c>
-      <c r="Y46" t="s">
-        <v>90</v>
-      </c>
-      <c r="Z46" t="s">
-        <v>90</v>
-      </c>
-      <c r="AA46">
-        <v>3</v>
-      </c>
-      <c r="AB46">
-        <v>1</v>
-      </c>
-      <c r="AC46">
-        <v>3</v>
-      </c>
-      <c r="AD46">
-        <v>3</v>
-      </c>
-      <c r="AE46">
-        <v>0</v>
-      </c>
-      <c r="AF46">
-        <v>1</v>
-      </c>
-      <c r="AG46">
-        <v>7</v>
-      </c>
-      <c r="AH46">
-        <v>5</v>
-      </c>
-      <c r="AI46">
-        <v>3</v>
-      </c>
-      <c r="AJ46">
-        <v>0</v>
-      </c>
-      <c r="AK46">
-        <v>0.67</v>
-      </c>
-      <c r="AL46">
-        <v>0.09</v>
-      </c>
-      <c r="AM46">
-        <v>0.48</v>
-      </c>
-      <c r="AN46">
-        <v>0.23</v>
-      </c>
-      <c r="AO46">
-        <v>1.1499999999999999</v>
-      </c>
-      <c r="AP46">
-        <v>0.32</v>
-      </c>
-      <c r="AQ46">
-        <v>1.37</v>
-      </c>
-      <c r="AR46">
-        <v>0.7</v>
-      </c>
-      <c r="AS46">
-        <v>427</v>
-      </c>
-      <c r="AT46">
-        <v>421</v>
-      </c>
-      <c r="AU46">
-        <v>230</v>
-      </c>
-      <c r="AV46">
-        <v>203</v>
-      </c>
-      <c r="AW46">
-        <v>104</v>
-      </c>
-      <c r="AX46">
-        <v>125</v>
-      </c>
-      <c r="AY46">
-        <v>26</v>
-      </c>
-      <c r="AZ46">
-        <v>34</v>
-      </c>
-      <c r="BA46">
-        <v>3</v>
-      </c>
-      <c r="BB46">
-        <v>3</v>
-      </c>
-      <c r="BC46">
-        <v>24</v>
-      </c>
-      <c r="BD46">
-        <v>16</v>
-      </c>
-      <c r="BE46">
-        <v>16</v>
-      </c>
-      <c r="BF46">
-        <v>17</v>
-      </c>
-      <c r="BG46">
-        <v>0</v>
-      </c>
-      <c r="BH46">
-        <v>5</v>
-      </c>
-      <c r="BI46" t="s">
-        <v>90</v>
-      </c>
-      <c r="BJ46" t="s">
-        <v>90</v>
-      </c>
-      <c r="BK46">
-        <v>15</v>
-      </c>
-      <c r="BL46">
-        <v>17</v>
-      </c>
-      <c r="BM46">
-        <v>13</v>
-      </c>
-      <c r="BN46">
-        <v>16</v>
-      </c>
-      <c r="BO46">
-        <v>2</v>
-      </c>
-      <c r="BP46">
-        <v>3</v>
-      </c>
-      <c r="BQ46">
-        <v>24</v>
-      </c>
-      <c r="BR46">
-        <v>40</v>
-      </c>
-      <c r="BS46">
-        <v>0</v>
-      </c>
-      <c r="BT46">
-        <v>3</v>
-      </c>
-      <c r="BU46" t="s">
-        <v>90</v>
-      </c>
-      <c r="BV46" t="s">
-        <v>90</v>
-      </c>
-      <c r="BW46">
-        <v>62</v>
-      </c>
-      <c r="BX46">
-        <v>55</v>
-      </c>
-      <c r="BY46">
-        <v>37</v>
-      </c>
-      <c r="BZ46">
-        <v>29</v>
-      </c>
-      <c r="CA46">
-        <v>25</v>
-      </c>
-      <c r="CB46">
-        <v>26</v>
-      </c>
-      <c r="CC46">
-        <v>11</v>
-      </c>
-      <c r="CD46">
-        <v>1</v>
-      </c>
-      <c r="CE46" t="s">
-        <v>90</v>
-      </c>
-      <c r="CF46" t="s">
-        <v>90</v>
-      </c>
-      <c r="CG46">
-        <v>1</v>
-      </c>
-      <c r="CH46">
-        <v>1</v>
-      </c>
-      <c r="CI46">
-        <v>1</v>
-      </c>
-      <c r="CJ46">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47" spans="2:88" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="B47" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="C47" t="s">
-        <v>101</v>
-      </c>
-      <c r="D47" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="E47">
-        <v>1</v>
-      </c>
-      <c r="F47">
-        <v>0</v>
-      </c>
-      <c r="G47">
-        <v>56</v>
-      </c>
-      <c r="H47">
-        <f t="shared" si="0"/>
-        <v>44</v>
-      </c>
-      <c r="I47">
-        <v>1.8</v>
-      </c>
-      <c r="J47">
-        <v>0.8</v>
-      </c>
-      <c r="K47">
-        <v>15</v>
-      </c>
-      <c r="L47">
-        <v>9</v>
-      </c>
-      <c r="M47">
-        <v>7</v>
-      </c>
-      <c r="N47">
-        <v>3</v>
-      </c>
-      <c r="O47">
-        <v>3</v>
-      </c>
-      <c r="P47">
-        <v>2</v>
-      </c>
-      <c r="Q47">
-        <v>3</v>
-      </c>
-      <c r="R47">
-        <v>2</v>
-      </c>
-      <c r="S47">
-        <v>360</v>
-      </c>
-      <c r="T47">
-        <v>270</v>
-      </c>
-      <c r="U47">
-        <v>8</v>
-      </c>
-      <c r="V47">
-        <v>17</v>
-      </c>
-      <c r="W47">
-        <v>7</v>
-      </c>
-      <c r="X47">
-        <v>3</v>
-      </c>
-      <c r="Y47" t="s">
-        <v>90</v>
-      </c>
-      <c r="Z47" t="s">
-        <v>90</v>
-      </c>
-      <c r="AA47">
-        <v>4</v>
-      </c>
-      <c r="AB47">
-        <v>2</v>
-      </c>
-      <c r="AC47">
-        <v>4</v>
-      </c>
-      <c r="AD47">
-        <v>4</v>
-      </c>
-      <c r="AE47">
-        <v>0</v>
-      </c>
-      <c r="AF47">
-        <v>0</v>
-      </c>
-      <c r="AG47">
-        <v>11</v>
-      </c>
-      <c r="AH47">
-        <v>7</v>
-      </c>
-      <c r="AI47">
-        <v>4</v>
-      </c>
-      <c r="AJ47">
-        <v>2</v>
-      </c>
-      <c r="AK47">
-        <v>1.53</v>
-      </c>
-      <c r="AL47">
-        <v>0.5</v>
-      </c>
-      <c r="AM47">
-        <v>0.27</v>
-      </c>
-      <c r="AN47">
-        <v>0.3</v>
-      </c>
-      <c r="AO47">
-        <v>1.8</v>
-      </c>
-      <c r="AP47">
-        <v>0.8</v>
-      </c>
-      <c r="AQ47">
-        <v>1.78</v>
-      </c>
-      <c r="AR47">
-        <v>1.1399999999999999</v>
-      </c>
-      <c r="AS47">
-        <v>449</v>
-      </c>
-      <c r="AT47">
-        <v>360</v>
-      </c>
-      <c r="AU47">
-        <v>169</v>
-      </c>
-      <c r="AV47">
-        <v>133</v>
-      </c>
-      <c r="AW47">
-        <v>191</v>
-      </c>
-      <c r="AX47">
-        <v>137</v>
-      </c>
-      <c r="AY47">
-        <v>24</v>
-      </c>
-      <c r="AZ47">
-        <v>19</v>
-      </c>
-      <c r="BA47">
-        <v>5</v>
-      </c>
-      <c r="BB47">
-        <v>1</v>
-      </c>
-      <c r="BC47">
-        <v>31</v>
-      </c>
-      <c r="BD47">
-        <v>28</v>
-      </c>
-      <c r="BE47">
-        <v>28</v>
-      </c>
-      <c r="BF47">
-        <v>22</v>
-      </c>
-      <c r="BG47">
-        <v>1</v>
-      </c>
-      <c r="BH47">
-        <v>0</v>
-      </c>
-      <c r="BI47" t="s">
-        <v>90</v>
-      </c>
-      <c r="BJ47" t="s">
-        <v>90</v>
-      </c>
-      <c r="BK47">
-        <v>22</v>
-      </c>
-      <c r="BL47">
-        <v>29</v>
-      </c>
-      <c r="BM47">
-        <v>12</v>
-      </c>
-      <c r="BN47">
-        <v>12</v>
-      </c>
-      <c r="BO47">
-        <v>4</v>
-      </c>
-      <c r="BP47">
-        <v>4</v>
-      </c>
-      <c r="BQ47">
-        <v>27</v>
-      </c>
-      <c r="BR47">
-        <v>31</v>
-      </c>
-      <c r="BS47">
-        <v>3</v>
-      </c>
-      <c r="BT47">
-        <v>6</v>
-      </c>
-      <c r="BU47" t="s">
-        <v>90</v>
-      </c>
-      <c r="BV47" t="s">
-        <v>90</v>
-      </c>
-      <c r="BW47">
-        <v>70</v>
-      </c>
-      <c r="BX47">
-        <v>59</v>
-      </c>
-      <c r="BY47">
-        <v>46</v>
-      </c>
-      <c r="BZ47">
-        <v>38</v>
-      </c>
-      <c r="CA47">
-        <v>24</v>
-      </c>
-      <c r="CB47">
-        <v>21</v>
-      </c>
-      <c r="CC47">
-        <v>9</v>
-      </c>
-      <c r="CD47">
-        <v>3</v>
-      </c>
-      <c r="CE47" t="s">
-        <v>90</v>
-      </c>
-      <c r="CF47" t="s">
-        <v>90</v>
-      </c>
-      <c r="CG47">
-        <v>2</v>
-      </c>
-      <c r="CH47">
-        <v>2</v>
-      </c>
-      <c r="CI47">
-        <v>0</v>
-      </c>
-      <c r="CJ47">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Oct 18, 2026, 10:32 PM
</commit_message>
<xml_diff>
--- a/Bundesliga 26-27.xlsx
+++ b/Bundesliga 26-27.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kuba\Desktop\analityczka\26-27\Bundesliga 26-27\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kuba\Desktop\analityczka\26-27\Ekstraklasa 26-27\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A8EA9779-D062-4EAD-93A3-716C256C24CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CAB22DA5-72E4-4F3E-9CD6-2FFC756BA321}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{723BE2C8-720D-41E0-A496-B3B96A8488E1}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="560" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="582" uniqueCount="131">
   <si>
     <t>date</t>
   </si>
@@ -426,6 +426,12 @@
   </si>
   <si>
     <t>Sat 17 October, 18:30</t>
+  </si>
+  <si>
+    <t>Sun 18 October, 15:30</t>
+  </si>
+  <si>
+    <t>Sun 18 October, 17:30</t>
   </si>
 </sst>
 </file>
@@ -843,7 +849,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9ED51FE2-0441-4690-9385-28E7CF18BF79}">
-  <dimension ref="B1:CJ44"/>
+  <dimension ref="B1:CJ46"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="17.7109375" customWidth="1"/>
@@ -1164,7 +1170,7 @@
         <v>59</v>
       </c>
       <c r="H2">
-        <f t="shared" ref="H2:H44" si="0">100-G2</f>
+        <f t="shared" ref="H2:H46" si="0">100-G2</f>
         <v>41</v>
       </c>
       <c r="I2">
@@ -12493,6 +12499,534 @@
         <v>0</v>
       </c>
       <c r="CJ44">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="2:88" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B45" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="D45" t="s">
+        <v>106</v>
+      </c>
+      <c r="E45">
+        <v>2</v>
+      </c>
+      <c r="F45">
+        <v>1</v>
+      </c>
+      <c r="G45">
+        <v>49</v>
+      </c>
+      <c r="H45">
+        <f t="shared" si="0"/>
+        <v>51</v>
+      </c>
+      <c r="I45">
+        <v>1.63</v>
+      </c>
+      <c r="J45">
+        <v>1.06</v>
+      </c>
+      <c r="K45">
+        <v>12</v>
+      </c>
+      <c r="L45">
+        <v>11</v>
+      </c>
+      <c r="M45">
+        <v>5</v>
+      </c>
+      <c r="N45">
+        <v>2</v>
+      </c>
+      <c r="O45">
+        <v>3</v>
+      </c>
+      <c r="P45">
+        <v>2</v>
+      </c>
+      <c r="Q45">
+        <v>1</v>
+      </c>
+      <c r="R45">
+        <v>1</v>
+      </c>
+      <c r="S45">
+        <v>416</v>
+      </c>
+      <c r="T45">
+        <v>432</v>
+      </c>
+      <c r="U45">
+        <v>12</v>
+      </c>
+      <c r="V45">
+        <v>5</v>
+      </c>
+      <c r="W45">
+        <v>4</v>
+      </c>
+      <c r="X45">
+        <v>3</v>
+      </c>
+      <c r="Y45" t="s">
+        <v>90</v>
+      </c>
+      <c r="Z45" t="s">
+        <v>90</v>
+      </c>
+      <c r="AA45">
+        <v>4</v>
+      </c>
+      <c r="AB45">
+        <v>8</v>
+      </c>
+      <c r="AC45">
+        <v>3</v>
+      </c>
+      <c r="AD45">
+        <v>1</v>
+      </c>
+      <c r="AE45">
+        <v>0</v>
+      </c>
+      <c r="AF45">
+        <v>0</v>
+      </c>
+      <c r="AG45">
+        <v>7</v>
+      </c>
+      <c r="AH45">
+        <v>8</v>
+      </c>
+      <c r="AI45">
+        <v>5</v>
+      </c>
+      <c r="AJ45">
+        <v>3</v>
+      </c>
+      <c r="AK45">
+        <v>1.52</v>
+      </c>
+      <c r="AL45">
+        <v>0.75</v>
+      </c>
+      <c r="AM45">
+        <v>0.1</v>
+      </c>
+      <c r="AN45">
+        <v>0.31</v>
+      </c>
+      <c r="AO45">
+        <v>1.63</v>
+      </c>
+      <c r="AP45">
+        <v>1.06</v>
+      </c>
+      <c r="AQ45">
+        <v>1.66</v>
+      </c>
+      <c r="AR45">
+        <v>0.71</v>
+      </c>
+      <c r="AS45">
+        <v>488</v>
+      </c>
+      <c r="AT45">
+        <v>508</v>
+      </c>
+      <c r="AU45">
+        <v>243</v>
+      </c>
+      <c r="AV45">
+        <v>230</v>
+      </c>
+      <c r="AW45">
+        <v>173</v>
+      </c>
+      <c r="AX45">
+        <v>202</v>
+      </c>
+      <c r="AY45">
+        <v>31</v>
+      </c>
+      <c r="AZ45">
+        <v>16</v>
+      </c>
+      <c r="BA45">
+        <v>0</v>
+      </c>
+      <c r="BB45">
+        <v>7</v>
+      </c>
+      <c r="BC45">
+        <v>16</v>
+      </c>
+      <c r="BD45">
+        <v>17</v>
+      </c>
+      <c r="BE45">
+        <v>16</v>
+      </c>
+      <c r="BF45">
+        <v>20</v>
+      </c>
+      <c r="BG45">
+        <v>1</v>
+      </c>
+      <c r="BH45">
+        <v>0</v>
+      </c>
+      <c r="BI45" t="s">
+        <v>90</v>
+      </c>
+      <c r="BJ45" t="s">
+        <v>90</v>
+      </c>
+      <c r="BK45">
+        <v>18</v>
+      </c>
+      <c r="BL45">
+        <v>13</v>
+      </c>
+      <c r="BM45">
+        <v>3</v>
+      </c>
+      <c r="BN45">
+        <v>12</v>
+      </c>
+      <c r="BO45">
+        <v>1</v>
+      </c>
+      <c r="BP45">
+        <v>3</v>
+      </c>
+      <c r="BQ45">
+        <v>26</v>
+      </c>
+      <c r="BR45">
+        <v>26</v>
+      </c>
+      <c r="BS45">
+        <v>1</v>
+      </c>
+      <c r="BT45">
+        <v>3</v>
+      </c>
+      <c r="BU45" t="s">
+        <v>90</v>
+      </c>
+      <c r="BV45" t="s">
+        <v>90</v>
+      </c>
+      <c r="BW45">
+        <v>35</v>
+      </c>
+      <c r="BX45">
+        <v>46</v>
+      </c>
+      <c r="BY45">
+        <v>28</v>
+      </c>
+      <c r="BZ45">
+        <v>31</v>
+      </c>
+      <c r="CA45">
+        <v>7</v>
+      </c>
+      <c r="CB45">
+        <v>15</v>
+      </c>
+      <c r="CC45">
+        <v>5</v>
+      </c>
+      <c r="CD45">
+        <v>6</v>
+      </c>
+      <c r="CE45" t="s">
+        <v>90</v>
+      </c>
+      <c r="CF45" t="s">
+        <v>90</v>
+      </c>
+      <c r="CG45">
+        <v>0</v>
+      </c>
+      <c r="CH45">
+        <v>1</v>
+      </c>
+      <c r="CI45">
+        <v>0</v>
+      </c>
+      <c r="CJ45">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="2:88" ht="30" x14ac:dyDescent="0.25">
+      <c r="B46" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="D46" t="s">
+        <v>95</v>
+      </c>
+      <c r="E46">
+        <v>1</v>
+      </c>
+      <c r="F46">
+        <v>2</v>
+      </c>
+      <c r="G46">
+        <v>48</v>
+      </c>
+      <c r="H46">
+        <f t="shared" si="0"/>
+        <v>52</v>
+      </c>
+      <c r="I46">
+        <v>0.34</v>
+      </c>
+      <c r="J46">
+        <v>1.78</v>
+      </c>
+      <c r="K46">
+        <v>9</v>
+      </c>
+      <c r="L46">
+        <v>14</v>
+      </c>
+      <c r="M46">
+        <v>3</v>
+      </c>
+      <c r="N46">
+        <v>8</v>
+      </c>
+      <c r="O46">
+        <v>0</v>
+      </c>
+      <c r="P46">
+        <v>3</v>
+      </c>
+      <c r="Q46">
+        <v>0</v>
+      </c>
+      <c r="R46">
+        <v>2</v>
+      </c>
+      <c r="S46">
+        <v>310</v>
+      </c>
+      <c r="T46">
+        <v>343</v>
+      </c>
+      <c r="U46">
+        <v>13</v>
+      </c>
+      <c r="V46">
+        <v>13</v>
+      </c>
+      <c r="W46">
+        <v>3</v>
+      </c>
+      <c r="X46">
+        <v>6</v>
+      </c>
+      <c r="Y46" t="s">
+        <v>90</v>
+      </c>
+      <c r="Z46" t="s">
+        <v>90</v>
+      </c>
+      <c r="AA46">
+        <v>3</v>
+      </c>
+      <c r="AB46">
+        <v>3</v>
+      </c>
+      <c r="AC46">
+        <v>3</v>
+      </c>
+      <c r="AD46">
+        <v>3</v>
+      </c>
+      <c r="AE46">
+        <v>0</v>
+      </c>
+      <c r="AF46">
+        <v>2</v>
+      </c>
+      <c r="AG46">
+        <v>4</v>
+      </c>
+      <c r="AH46">
+        <v>9</v>
+      </c>
+      <c r="AI46">
+        <v>5</v>
+      </c>
+      <c r="AJ46">
+        <v>5</v>
+      </c>
+      <c r="AK46">
+        <v>0.3</v>
+      </c>
+      <c r="AL46">
+        <v>1.49</v>
+      </c>
+      <c r="AM46">
+        <v>0.04</v>
+      </c>
+      <c r="AN46">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="AO46">
+        <v>0.34</v>
+      </c>
+      <c r="AP46">
+        <v>1.78</v>
+      </c>
+      <c r="AQ46">
+        <v>1.18</v>
+      </c>
+      <c r="AR46">
+        <v>2.41</v>
+      </c>
+      <c r="AS46">
+        <v>397</v>
+      </c>
+      <c r="AT46">
+        <v>441</v>
+      </c>
+      <c r="AU46">
+        <v>199</v>
+      </c>
+      <c r="AV46">
+        <v>167</v>
+      </c>
+      <c r="AW46">
+        <v>111</v>
+      </c>
+      <c r="AX46">
+        <v>176</v>
+      </c>
+      <c r="AY46">
+        <v>21</v>
+      </c>
+      <c r="AZ46">
+        <v>23</v>
+      </c>
+      <c r="BA46">
+        <v>0</v>
+      </c>
+      <c r="BB46">
+        <v>3</v>
+      </c>
+      <c r="BC46">
+        <v>25</v>
+      </c>
+      <c r="BD46">
+        <v>21</v>
+      </c>
+      <c r="BE46">
+        <v>19</v>
+      </c>
+      <c r="BF46">
+        <v>34</v>
+      </c>
+      <c r="BG46">
+        <v>3</v>
+      </c>
+      <c r="BH46">
+        <v>2</v>
+      </c>
+      <c r="BI46" t="s">
+        <v>90</v>
+      </c>
+      <c r="BJ46" t="s">
+        <v>90</v>
+      </c>
+      <c r="BK46">
+        <v>20</v>
+      </c>
+      <c r="BL46">
+        <v>15</v>
+      </c>
+      <c r="BM46">
+        <v>10</v>
+      </c>
+      <c r="BN46">
+        <v>7</v>
+      </c>
+      <c r="BO46">
+        <v>3</v>
+      </c>
+      <c r="BP46">
+        <v>3</v>
+      </c>
+      <c r="BQ46">
+        <v>46</v>
+      </c>
+      <c r="BR46">
+        <v>31</v>
+      </c>
+      <c r="BS46">
+        <v>6</v>
+      </c>
+      <c r="BT46">
+        <v>2</v>
+      </c>
+      <c r="BU46" t="s">
+        <v>90</v>
+      </c>
+      <c r="BV46" t="s">
+        <v>90</v>
+      </c>
+      <c r="BW46">
+        <v>61</v>
+      </c>
+      <c r="BX46">
+        <v>71</v>
+      </c>
+      <c r="BY46">
+        <v>37</v>
+      </c>
+      <c r="BZ46">
+        <v>39</v>
+      </c>
+      <c r="CA46">
+        <v>24</v>
+      </c>
+      <c r="CB46">
+        <v>22</v>
+      </c>
+      <c r="CC46">
+        <v>5</v>
+      </c>
+      <c r="CD46">
+        <v>12</v>
+      </c>
+      <c r="CE46" t="s">
+        <v>90</v>
+      </c>
+      <c r="CF46" t="s">
+        <v>90</v>
+      </c>
+      <c r="CG46">
+        <v>3</v>
+      </c>
+      <c r="CH46">
+        <v>2</v>
+      </c>
+      <c r="CI46">
+        <v>0</v>
+      </c>
+      <c r="CJ46">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Oct 24, 2026, 10:31 PM
</commit_message>
<xml_diff>
--- a/Bundesliga 26-27.xlsx
+++ b/Bundesliga 26-27.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kuba\Desktop\analityczka\26-27\Ekstraklasa 26-27\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CAB22DA5-72E4-4F3E-9CD6-2FFC756BA321}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8F49A4A4-19EC-4255-B6E3-918109945DFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{723BE2C8-720D-41E0-A496-B3B96A8488E1}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="582" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="593" uniqueCount="132">
   <si>
     <t>date</t>
   </si>
@@ -433,12 +433,15 @@
   <si>
     <t>Sun 18 October, 17:30</t>
   </si>
+  <si>
+    <t>Fri 23 October, 20:30</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -474,6 +477,11 @@
       <family val="2"/>
       <charset val="238"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Inherit"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -495,7 +503,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
@@ -514,6 +522,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -849,8 +860,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9ED51FE2-0441-4690-9385-28E7CF18BF79}">
-  <dimension ref="B1:CJ46"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="B1:CJ47"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="17.7109375" customWidth="1"/>
     <col min="3" max="3" width="19" customWidth="1"/>
@@ -887,7 +898,7 @@
     <col min="84" max="84" width="11.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:88" ht="75" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:88" ht="75">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1150,7 +1161,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="2" spans="2:88" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:88" ht="28.5" customHeight="1">
       <c r="B2" s="3" t="s">
         <v>89</v>
       </c>
@@ -1170,7 +1181,7 @@
         <v>59</v>
       </c>
       <c r="H2">
-        <f t="shared" ref="H2:H46" si="0">100-G2</f>
+        <f t="shared" ref="H2:H47" si="0">100-G2</f>
         <v>41</v>
       </c>
       <c r="I2">
@@ -1414,7 +1425,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:88" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:88" ht="25.5" customHeight="1">
       <c r="B3" s="3" t="s">
         <v>91</v>
       </c>
@@ -1678,7 +1689,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="2:88" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:88" ht="21.75" customHeight="1">
       <c r="B4" s="3" t="s">
         <v>91</v>
       </c>
@@ -1942,7 +1953,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="2:88" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:88" ht="24.75" customHeight="1">
       <c r="B5" s="3" t="s">
         <v>91</v>
       </c>
@@ -2206,7 +2217,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="2:88" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:88" ht="24" customHeight="1">
       <c r="B6" s="3" t="s">
         <v>91</v>
       </c>
@@ -2470,7 +2481,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="2:88" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:88" ht="30" customHeight="1">
       <c r="B7" s="3" t="s">
         <v>91</v>
       </c>
@@ -2734,7 +2745,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="2:88" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:88" ht="27.75" customHeight="1">
       <c r="B8" s="3" t="s">
         <v>102</v>
       </c>
@@ -2998,7 +3009,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="2:88" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:88" ht="27" customHeight="1">
       <c r="B9" s="3" t="s">
         <v>105</v>
       </c>
@@ -3262,7 +3273,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="2:88" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:88" ht="30.75" customHeight="1">
       <c r="B10" s="3" t="s">
         <v>105</v>
       </c>
@@ -3526,7 +3537,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="2:88" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:88" ht="24.75" customHeight="1">
       <c r="B11" s="3" t="s">
         <v>110</v>
       </c>
@@ -3790,7 +3801,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="2:88" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:88" ht="25.5">
       <c r="B12" s="3" t="s">
         <v>111</v>
       </c>
@@ -4054,7 +4065,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="2:88" ht="30" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:88" ht="30">
       <c r="B13" s="3" t="s">
         <v>111</v>
       </c>
@@ -4318,7 +4329,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="2:88" ht="30" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:88" ht="30">
       <c r="B14" s="3" t="s">
         <v>111</v>
       </c>
@@ -4582,7 +4593,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="2:88" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:88" ht="25.5">
       <c r="B15" s="3" t="s">
         <v>111</v>
       </c>
@@ -4846,7 +4857,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="2:88" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:88" ht="25.5">
       <c r="B16" s="3" t="s">
         <v>111</v>
       </c>
@@ -5110,7 +5121,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="2:88" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:88" ht="25.5">
       <c r="B17" s="3" t="s">
         <v>112</v>
       </c>
@@ -5374,7 +5385,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="2:88" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:88" ht="25.5">
       <c r="B18" s="3" t="s">
         <v>113</v>
       </c>
@@ -5638,7 +5649,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="2:88" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:88" ht="25.5">
       <c r="B19" s="3" t="s">
         <v>114</v>
       </c>
@@ -5902,7 +5913,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="2:88" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:88" ht="25.5">
       <c r="B20" s="3" t="s">
         <v>115</v>
       </c>
@@ -6166,7 +6177,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="2:88" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:88" ht="25.5">
       <c r="B21" s="3" t="s">
         <v>116</v>
       </c>
@@ -6430,7 +6441,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="2:88" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:88" ht="25.5">
       <c r="B22" s="3" t="s">
         <v>116</v>
       </c>
@@ -6694,7 +6705,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="2:88" ht="30" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:88" ht="30">
       <c r="B23" s="3" t="s">
         <v>116</v>
       </c>
@@ -6958,7 +6969,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="2:88" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:88" ht="25.5">
       <c r="B24" s="3" t="s">
         <v>116</v>
       </c>
@@ -7222,7 +7233,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="2:88" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:88" ht="25.5">
       <c r="B25" s="3" t="s">
         <v>116</v>
       </c>
@@ -7486,7 +7497,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="2:88" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:88" ht="25.5">
       <c r="B26" s="3" t="s">
         <v>117</v>
       </c>
@@ -7750,7 +7761,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="2:88" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:88" ht="25.5">
       <c r="B27" s="3" t="s">
         <v>118</v>
       </c>
@@ -8014,7 +8025,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="2:88" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:88" ht="25.5">
       <c r="B28" s="3" t="s">
         <v>119</v>
       </c>
@@ -8278,7 +8289,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="2:88" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:88" ht="25.5">
       <c r="B29" s="3" t="s">
         <v>120</v>
       </c>
@@ -8542,7 +8553,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="2:88" ht="30" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:88" ht="30">
       <c r="B30" s="3" t="s">
         <v>121</v>
       </c>
@@ -8806,7 +8817,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="2:88" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:88" ht="25.5">
       <c r="B31" s="3" t="s">
         <v>121</v>
       </c>
@@ -9070,7 +9081,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="2:88" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:88" ht="25.5">
       <c r="B32" s="3" t="s">
         <v>121</v>
       </c>
@@ -9334,7 +9345,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="2:88" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:88" ht="25.5">
       <c r="B33" s="3" t="s">
         <v>121</v>
       </c>
@@ -9598,7 +9609,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="2:88" ht="30" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:88" ht="30">
       <c r="B34" s="3" t="s">
         <v>122</v>
       </c>
@@ -9862,7 +9873,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="2:88" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:88" ht="25.5">
       <c r="B35" s="3" t="s">
         <v>123</v>
       </c>
@@ -10126,7 +10137,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="2:88" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:88" ht="25.5">
       <c r="B36" s="3" t="s">
         <v>124</v>
       </c>
@@ -10390,7 +10401,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="2:88" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:88" ht="25.5">
       <c r="B37" s="3" t="s">
         <v>125</v>
       </c>
@@ -10654,7 +10665,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="2:88" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:88">
       <c r="B38" s="6" t="s">
         <v>126</v>
       </c>
@@ -10918,7 +10929,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="2:88" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:88" ht="25.5">
       <c r="B39" s="3" t="s">
         <v>127</v>
       </c>
@@ -11182,7 +11193,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="2:88" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:88" ht="25.5">
       <c r="B40" s="3" t="s">
         <v>127</v>
       </c>
@@ -11446,7 +11457,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="2:88" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:88" ht="25.5">
       <c r="B41" s="3" t="s">
         <v>127</v>
       </c>
@@ -11710,7 +11721,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="2:88" ht="30" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:88" ht="30">
       <c r="B42" s="3" t="s">
         <v>127</v>
       </c>
@@ -11974,7 +11985,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="2:88" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:88" ht="25.5">
       <c r="B43" s="3" t="s">
         <v>127</v>
       </c>
@@ -12238,7 +12249,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="2:88" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:88" ht="25.5">
       <c r="B44" s="3" t="s">
         <v>128</v>
       </c>
@@ -12502,7 +12513,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="2:88" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:88" ht="25.5">
       <c r="B45" s="3" t="s">
         <v>129</v>
       </c>
@@ -12766,7 +12777,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="2:88" ht="30" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:88" ht="30">
       <c r="B46" s="3" t="s">
         <v>130</v>
       </c>
@@ -13027,6 +13038,270 @@
         <v>0</v>
       </c>
       <c r="CJ46">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="2:88" ht="30">
+      <c r="B47" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="C47" t="s">
+        <v>88</v>
+      </c>
+      <c r="D47" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="E47">
+        <v>2</v>
+      </c>
+      <c r="F47">
+        <v>3</v>
+      </c>
+      <c r="G47">
+        <v>70</v>
+      </c>
+      <c r="H47">
+        <f t="shared" si="0"/>
+        <v>30</v>
+      </c>
+      <c r="I47">
+        <v>1.53</v>
+      </c>
+      <c r="J47">
+        <v>2.6</v>
+      </c>
+      <c r="K47">
+        <v>15</v>
+      </c>
+      <c r="L47">
+        <v>16</v>
+      </c>
+      <c r="M47">
+        <v>5</v>
+      </c>
+      <c r="N47">
+        <v>6</v>
+      </c>
+      <c r="O47">
+        <v>2</v>
+      </c>
+      <c r="P47">
+        <v>4</v>
+      </c>
+      <c r="Q47">
+        <v>1</v>
+      </c>
+      <c r="R47">
+        <v>2</v>
+      </c>
+      <c r="S47">
+        <v>590</v>
+      </c>
+      <c r="T47">
+        <v>189</v>
+      </c>
+      <c r="U47">
+        <v>9</v>
+      </c>
+      <c r="V47">
+        <v>14</v>
+      </c>
+      <c r="W47">
+        <v>6</v>
+      </c>
+      <c r="X47">
+        <v>5</v>
+      </c>
+      <c r="Y47" t="s">
+        <v>90</v>
+      </c>
+      <c r="Z47" t="s">
+        <v>90</v>
+      </c>
+      <c r="AA47">
+        <v>8</v>
+      </c>
+      <c r="AB47">
+        <v>7</v>
+      </c>
+      <c r="AC47">
+        <v>2</v>
+      </c>
+      <c r="AD47">
+        <v>3</v>
+      </c>
+      <c r="AE47">
+        <v>0</v>
+      </c>
+      <c r="AF47">
+        <v>1</v>
+      </c>
+      <c r="AG47">
+        <v>10</v>
+      </c>
+      <c r="AH47">
+        <v>12</v>
+      </c>
+      <c r="AI47">
+        <v>5</v>
+      </c>
+      <c r="AJ47">
+        <v>4</v>
+      </c>
+      <c r="AK47">
+        <v>1.2</v>
+      </c>
+      <c r="AL47">
+        <v>2.12</v>
+      </c>
+      <c r="AM47">
+        <v>0.33</v>
+      </c>
+      <c r="AN47">
+        <v>0.48</v>
+      </c>
+      <c r="AO47">
+        <v>1.53</v>
+      </c>
+      <c r="AP47">
+        <v>2.6</v>
+      </c>
+      <c r="AQ47">
+        <v>1.69</v>
+      </c>
+      <c r="AR47">
+        <v>2.67</v>
+      </c>
+      <c r="AS47">
+        <v>691</v>
+      </c>
+      <c r="AT47">
+        <v>288</v>
+      </c>
+      <c r="AU47">
+        <v>285</v>
+      </c>
+      <c r="AV47">
+        <v>110</v>
+      </c>
+      <c r="AW47">
+        <v>305</v>
+      </c>
+      <c r="AX47">
+        <v>79</v>
+      </c>
+      <c r="AY47">
+        <v>25</v>
+      </c>
+      <c r="AZ47">
+        <v>11</v>
+      </c>
+      <c r="BA47">
+        <v>8</v>
+      </c>
+      <c r="BB47">
+        <v>2</v>
+      </c>
+      <c r="BC47">
+        <v>22</v>
+      </c>
+      <c r="BD47">
+        <v>11</v>
+      </c>
+      <c r="BE47">
+        <v>26</v>
+      </c>
+      <c r="BF47">
+        <v>21</v>
+      </c>
+      <c r="BG47">
+        <v>2</v>
+      </c>
+      <c r="BH47">
+        <v>2</v>
+      </c>
+      <c r="BI47" t="s">
+        <v>90</v>
+      </c>
+      <c r="BJ47" t="s">
+        <v>90</v>
+      </c>
+      <c r="BK47">
+        <v>4</v>
+      </c>
+      <c r="BL47">
+        <v>11</v>
+      </c>
+      <c r="BM47">
+        <v>10</v>
+      </c>
+      <c r="BN47">
+        <v>17</v>
+      </c>
+      <c r="BO47">
+        <v>3</v>
+      </c>
+      <c r="BP47">
+        <v>1</v>
+      </c>
+      <c r="BQ47">
+        <v>24</v>
+      </c>
+      <c r="BR47">
+        <v>30</v>
+      </c>
+      <c r="BS47">
+        <v>2</v>
+      </c>
+      <c r="BT47">
+        <v>3</v>
+      </c>
+      <c r="BU47" t="s">
+        <v>90</v>
+      </c>
+      <c r="BV47" t="s">
+        <v>90</v>
+      </c>
+      <c r="BW47">
+        <v>51</v>
+      </c>
+      <c r="BX47">
+        <v>43</v>
+      </c>
+      <c r="BY47">
+        <v>23</v>
+      </c>
+      <c r="BZ47">
+        <v>24</v>
+      </c>
+      <c r="CA47">
+        <v>28</v>
+      </c>
+      <c r="CB47">
+        <v>19</v>
+      </c>
+      <c r="CC47">
+        <v>6</v>
+      </c>
+      <c r="CD47">
+        <v>5</v>
+      </c>
+      <c r="CE47" t="s">
+        <v>90</v>
+      </c>
+      <c r="CF47" t="s">
+        <v>90</v>
+      </c>
+      <c r="CG47">
+        <v>2</v>
+      </c>
+      <c r="CH47">
+        <v>4</v>
+      </c>
+      <c r="CI47">
+        <v>0</v>
+      </c>
+      <c r="CJ47">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Oct 25, 2026, 11:28 AM
</commit_message>
<xml_diff>
--- a/Bundesliga 26-27.xlsx
+++ b/Bundesliga 26-27.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kuba\Desktop\analityczka\26-27\Ekstraklasa 26-27\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8F49A4A4-19EC-4255-B6E3-918109945DFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{750824C8-E38B-4868-B529-6B406F92FDA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{723BE2C8-720D-41E0-A496-B3B96A8488E1}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="593" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="659" uniqueCount="134">
   <si>
     <t>date</t>
   </si>
@@ -435,6 +435,12 @@
   </si>
   <si>
     <t>Fri 23 October, 20:30</t>
+  </si>
+  <si>
+    <t>Sat 24 October, 15:30</t>
+  </si>
+  <si>
+    <t>Sat 24 October, 18:30</t>
   </si>
 </sst>
 </file>
@@ -860,7 +866,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9ED51FE2-0441-4690-9385-28E7CF18BF79}">
-  <dimension ref="B1:CJ47"/>
+  <dimension ref="B1:CJ53"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="17.7109375" customWidth="1"/>
@@ -1181,7 +1187,7 @@
         <v>59</v>
       </c>
       <c r="H2">
-        <f t="shared" ref="H2:H47" si="0">100-G2</f>
+        <f t="shared" ref="H2:H53" si="0">100-G2</f>
         <v>41</v>
       </c>
       <c r="I2">
@@ -13302,6 +13308,1590 @@
         <v>0</v>
       </c>
       <c r="CJ47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="2:88" ht="25.5">
+      <c r="B48" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="C48" t="s">
+        <v>108</v>
+      </c>
+      <c r="D48" t="s">
+        <v>100</v>
+      </c>
+      <c r="E48">
+        <v>1</v>
+      </c>
+      <c r="F48">
+        <v>1</v>
+      </c>
+      <c r="G48">
+        <v>66</v>
+      </c>
+      <c r="H48">
+        <f t="shared" si="0"/>
+        <v>34</v>
+      </c>
+      <c r="I48">
+        <v>1.92</v>
+      </c>
+      <c r="J48">
+        <v>1.25</v>
+      </c>
+      <c r="K48">
+        <v>27</v>
+      </c>
+      <c r="L48">
+        <v>6</v>
+      </c>
+      <c r="M48">
+        <v>5</v>
+      </c>
+      <c r="N48">
+        <v>1</v>
+      </c>
+      <c r="O48">
+        <v>2</v>
+      </c>
+      <c r="P48">
+        <v>1</v>
+      </c>
+      <c r="Q48">
+        <v>2</v>
+      </c>
+      <c r="R48">
+        <v>0</v>
+      </c>
+      <c r="S48">
+        <v>520</v>
+      </c>
+      <c r="T48">
+        <v>224</v>
+      </c>
+      <c r="U48">
+        <v>10</v>
+      </c>
+      <c r="V48">
+        <v>9</v>
+      </c>
+      <c r="W48">
+        <v>5</v>
+      </c>
+      <c r="X48">
+        <v>1</v>
+      </c>
+      <c r="Y48" t="s">
+        <v>90</v>
+      </c>
+      <c r="Z48" t="s">
+        <v>90</v>
+      </c>
+      <c r="AA48">
+        <v>15</v>
+      </c>
+      <c r="AB48">
+        <v>1</v>
+      </c>
+      <c r="AC48">
+        <v>7</v>
+      </c>
+      <c r="AD48">
+        <v>4</v>
+      </c>
+      <c r="AE48">
+        <v>1</v>
+      </c>
+      <c r="AF48">
+        <v>0</v>
+      </c>
+      <c r="AG48">
+        <v>15</v>
+      </c>
+      <c r="AH48">
+        <v>3</v>
+      </c>
+      <c r="AI48">
+        <v>12</v>
+      </c>
+      <c r="AJ48">
+        <v>3</v>
+      </c>
+      <c r="AK48">
+        <v>1.45</v>
+      </c>
+      <c r="AL48">
+        <v>0.38</v>
+      </c>
+      <c r="AM48">
+        <v>0.47</v>
+      </c>
+      <c r="AN48">
+        <v>0.88</v>
+      </c>
+      <c r="AO48">
+        <v>1.92</v>
+      </c>
+      <c r="AP48">
+        <v>1.25</v>
+      </c>
+      <c r="AQ48">
+        <v>1.5</v>
+      </c>
+      <c r="AR48">
+        <v>0.99</v>
+      </c>
+      <c r="AS48">
+        <v>603</v>
+      </c>
+      <c r="AT48">
+        <v>316</v>
+      </c>
+      <c r="AU48">
+        <v>176</v>
+      </c>
+      <c r="AV48">
+        <v>149</v>
+      </c>
+      <c r="AW48">
+        <v>344</v>
+      </c>
+      <c r="AX48">
+        <v>75</v>
+      </c>
+      <c r="AY48">
+        <v>18</v>
+      </c>
+      <c r="AZ48">
+        <v>18</v>
+      </c>
+      <c r="BA48">
+        <v>12</v>
+      </c>
+      <c r="BB48">
+        <v>1</v>
+      </c>
+      <c r="BC48">
+        <v>28</v>
+      </c>
+      <c r="BD48">
+        <v>18</v>
+      </c>
+      <c r="BE48">
+        <v>41</v>
+      </c>
+      <c r="BF48">
+        <v>8</v>
+      </c>
+      <c r="BG48">
+        <v>0</v>
+      </c>
+      <c r="BH48">
+        <v>2</v>
+      </c>
+      <c r="BI48" t="s">
+        <v>90</v>
+      </c>
+      <c r="BJ48" t="s">
+        <v>90</v>
+      </c>
+      <c r="BK48">
+        <v>13</v>
+      </c>
+      <c r="BL48">
+        <v>10</v>
+      </c>
+      <c r="BM48">
+        <v>14</v>
+      </c>
+      <c r="BN48">
+        <v>7</v>
+      </c>
+      <c r="BO48">
+        <v>4</v>
+      </c>
+      <c r="BP48">
+        <v>7</v>
+      </c>
+      <c r="BQ48">
+        <v>16</v>
+      </c>
+      <c r="BR48">
+        <v>47</v>
+      </c>
+      <c r="BS48">
+        <v>0</v>
+      </c>
+      <c r="BT48">
+        <v>4</v>
+      </c>
+      <c r="BU48" t="s">
+        <v>90</v>
+      </c>
+      <c r="BV48" t="s">
+        <v>90</v>
+      </c>
+      <c r="BW48">
+        <v>41</v>
+      </c>
+      <c r="BX48">
+        <v>38</v>
+      </c>
+      <c r="BY48">
+        <v>23</v>
+      </c>
+      <c r="BZ48">
+        <v>20</v>
+      </c>
+      <c r="CA48">
+        <v>18</v>
+      </c>
+      <c r="CB48">
+        <v>18</v>
+      </c>
+      <c r="CC48">
+        <v>1</v>
+      </c>
+      <c r="CD48">
+        <v>3</v>
+      </c>
+      <c r="CE48" t="s">
+        <v>90</v>
+      </c>
+      <c r="CF48" t="s">
+        <v>90</v>
+      </c>
+      <c r="CG48">
+        <v>0</v>
+      </c>
+      <c r="CH48">
+        <v>3</v>
+      </c>
+      <c r="CI48">
+        <v>1</v>
+      </c>
+      <c r="CJ48">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="2:88" ht="25.5">
+      <c r="B49" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="D49" t="s">
+        <v>109</v>
+      </c>
+      <c r="E49">
+        <v>0</v>
+      </c>
+      <c r="F49">
+        <v>0</v>
+      </c>
+      <c r="G49">
+        <v>62</v>
+      </c>
+      <c r="H49">
+        <f t="shared" si="0"/>
+        <v>38</v>
+      </c>
+      <c r="I49">
+        <v>1.24</v>
+      </c>
+      <c r="J49">
+        <v>0.61</v>
+      </c>
+      <c r="K49">
+        <v>14</v>
+      </c>
+      <c r="L49">
+        <v>9</v>
+      </c>
+      <c r="M49">
+        <v>5</v>
+      </c>
+      <c r="N49">
+        <v>1</v>
+      </c>
+      <c r="O49">
+        <v>2</v>
+      </c>
+      <c r="P49">
+        <v>1</v>
+      </c>
+      <c r="Q49">
+        <v>2</v>
+      </c>
+      <c r="R49">
+        <v>1</v>
+      </c>
+      <c r="S49">
+        <v>455</v>
+      </c>
+      <c r="T49">
+        <v>225</v>
+      </c>
+      <c r="U49">
+        <v>8</v>
+      </c>
+      <c r="V49">
+        <v>12</v>
+      </c>
+      <c r="W49">
+        <v>6</v>
+      </c>
+      <c r="X49">
+        <v>5</v>
+      </c>
+      <c r="Y49" t="s">
+        <v>90</v>
+      </c>
+      <c r="Z49" t="s">
+        <v>90</v>
+      </c>
+      <c r="AA49">
+        <v>5</v>
+      </c>
+      <c r="AB49">
+        <v>6</v>
+      </c>
+      <c r="AC49">
+        <v>4</v>
+      </c>
+      <c r="AD49">
+        <v>2</v>
+      </c>
+      <c r="AE49">
+        <v>0</v>
+      </c>
+      <c r="AF49">
+        <v>1</v>
+      </c>
+      <c r="AG49">
+        <v>6</v>
+      </c>
+      <c r="AH49">
+        <v>8</v>
+      </c>
+      <c r="AI49">
+        <v>8</v>
+      </c>
+      <c r="AJ49">
+        <v>1</v>
+      </c>
+      <c r="AK49">
+        <v>1.23</v>
+      </c>
+      <c r="AL49">
+        <v>0.46</v>
+      </c>
+      <c r="AM49">
+        <v>0.01</v>
+      </c>
+      <c r="AN49">
+        <v>0.15</v>
+      </c>
+      <c r="AO49">
+        <v>1.24</v>
+      </c>
+      <c r="AP49">
+        <v>0.61</v>
+      </c>
+      <c r="AQ49">
+        <v>0.75</v>
+      </c>
+      <c r="AR49">
+        <v>0.26</v>
+      </c>
+      <c r="AS49">
+        <v>544</v>
+      </c>
+      <c r="AT49">
+        <v>322</v>
+      </c>
+      <c r="AU49">
+        <v>242</v>
+      </c>
+      <c r="AV49">
+        <v>87</v>
+      </c>
+      <c r="AW49">
+        <v>213</v>
+      </c>
+      <c r="AX49">
+        <v>138</v>
+      </c>
+      <c r="AY49">
+        <v>32</v>
+      </c>
+      <c r="AZ49">
+        <v>13</v>
+      </c>
+      <c r="BA49">
+        <v>2</v>
+      </c>
+      <c r="BB49">
+        <v>5</v>
+      </c>
+      <c r="BC49">
+        <v>24</v>
+      </c>
+      <c r="BD49">
+        <v>25</v>
+      </c>
+      <c r="BE49">
+        <v>28</v>
+      </c>
+      <c r="BF49">
+        <v>24</v>
+      </c>
+      <c r="BG49">
+        <v>4</v>
+      </c>
+      <c r="BH49">
+        <v>1</v>
+      </c>
+      <c r="BI49" t="s">
+        <v>90</v>
+      </c>
+      <c r="BJ49" t="s">
+        <v>90</v>
+      </c>
+      <c r="BK49">
+        <v>18</v>
+      </c>
+      <c r="BL49">
+        <v>25</v>
+      </c>
+      <c r="BM49">
+        <v>9</v>
+      </c>
+      <c r="BN49">
+        <v>13</v>
+      </c>
+      <c r="BO49">
+        <v>2</v>
+      </c>
+      <c r="BP49">
+        <v>5</v>
+      </c>
+      <c r="BQ49">
+        <v>43</v>
+      </c>
+      <c r="BR49">
+        <v>33</v>
+      </c>
+      <c r="BS49">
+        <v>1</v>
+      </c>
+      <c r="BT49">
+        <v>4</v>
+      </c>
+      <c r="BU49" t="s">
+        <v>90</v>
+      </c>
+      <c r="BV49" t="s">
+        <v>90</v>
+      </c>
+      <c r="BW49">
+        <v>63</v>
+      </c>
+      <c r="BX49">
+        <v>61</v>
+      </c>
+      <c r="BY49">
+        <v>39</v>
+      </c>
+      <c r="BZ49">
+        <v>41</v>
+      </c>
+      <c r="CA49">
+        <v>24</v>
+      </c>
+      <c r="CB49">
+        <v>20</v>
+      </c>
+      <c r="CC49">
+        <v>10</v>
+      </c>
+      <c r="CD49">
+        <v>8</v>
+      </c>
+      <c r="CE49" t="s">
+        <v>90</v>
+      </c>
+      <c r="CF49" t="s">
+        <v>90</v>
+      </c>
+      <c r="CG49">
+        <v>2</v>
+      </c>
+      <c r="CH49">
+        <v>3</v>
+      </c>
+      <c r="CI49">
+        <v>0</v>
+      </c>
+      <c r="CJ49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="2:88" ht="25.5">
+      <c r="B50" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="C50" t="s">
+        <v>96</v>
+      </c>
+      <c r="D50" t="s">
+        <v>107</v>
+      </c>
+      <c r="E50">
+        <v>2</v>
+      </c>
+      <c r="F50">
+        <v>3</v>
+      </c>
+      <c r="G50">
+        <v>54</v>
+      </c>
+      <c r="H50">
+        <f t="shared" si="0"/>
+        <v>46</v>
+      </c>
+      <c r="I50">
+        <v>1.7</v>
+      </c>
+      <c r="J50">
+        <v>2.69</v>
+      </c>
+      <c r="K50">
+        <v>18</v>
+      </c>
+      <c r="L50">
+        <v>17</v>
+      </c>
+      <c r="M50">
+        <v>8</v>
+      </c>
+      <c r="N50">
+        <v>8</v>
+      </c>
+      <c r="O50">
+        <v>4</v>
+      </c>
+      <c r="P50">
+        <v>3</v>
+      </c>
+      <c r="Q50">
+        <v>3</v>
+      </c>
+      <c r="R50">
+        <v>1</v>
+      </c>
+      <c r="S50">
+        <v>486</v>
+      </c>
+      <c r="T50">
+        <v>435</v>
+      </c>
+      <c r="U50">
+        <v>7</v>
+      </c>
+      <c r="V50">
+        <v>5</v>
+      </c>
+      <c r="W50">
+        <v>6</v>
+      </c>
+      <c r="X50">
+        <v>6</v>
+      </c>
+      <c r="Y50" t="s">
+        <v>90</v>
+      </c>
+      <c r="Z50" t="s">
+        <v>90</v>
+      </c>
+      <c r="AA50">
+        <v>7</v>
+      </c>
+      <c r="AB50">
+        <v>4</v>
+      </c>
+      <c r="AC50">
+        <v>3</v>
+      </c>
+      <c r="AD50">
+        <v>5</v>
+      </c>
+      <c r="AE50">
+        <v>0</v>
+      </c>
+      <c r="AF50">
+        <v>0</v>
+      </c>
+      <c r="AG50">
+        <v>15</v>
+      </c>
+      <c r="AH50">
+        <v>11</v>
+      </c>
+      <c r="AI50">
+        <v>3</v>
+      </c>
+      <c r="AJ50">
+        <v>6</v>
+      </c>
+      <c r="AK50">
+        <v>1.39</v>
+      </c>
+      <c r="AL50">
+        <v>0.62</v>
+      </c>
+      <c r="AM50">
+        <v>0.3</v>
+      </c>
+      <c r="AN50">
+        <v>0.49</v>
+      </c>
+      <c r="AO50">
+        <v>1.7</v>
+      </c>
+      <c r="AP50">
+        <v>1.1100000000000001</v>
+      </c>
+      <c r="AQ50">
+        <v>1.99</v>
+      </c>
+      <c r="AR50">
+        <v>2.71</v>
+      </c>
+      <c r="AS50">
+        <v>559</v>
+      </c>
+      <c r="AT50">
+        <v>505</v>
+      </c>
+      <c r="AU50">
+        <v>122</v>
+      </c>
+      <c r="AV50">
+        <v>273</v>
+      </c>
+      <c r="AW50">
+        <v>364</v>
+      </c>
+      <c r="AX50">
+        <v>162</v>
+      </c>
+      <c r="AY50">
+        <v>18</v>
+      </c>
+      <c r="AZ50">
+        <v>20</v>
+      </c>
+      <c r="BA50">
+        <v>14</v>
+      </c>
+      <c r="BB50">
+        <v>4</v>
+      </c>
+      <c r="BC50">
+        <v>19</v>
+      </c>
+      <c r="BD50">
+        <v>11</v>
+      </c>
+      <c r="BE50">
+        <v>45</v>
+      </c>
+      <c r="BF50">
+        <v>33</v>
+      </c>
+      <c r="BG50">
+        <v>2</v>
+      </c>
+      <c r="BH50">
+        <v>0</v>
+      </c>
+      <c r="BI50" t="s">
+        <v>90</v>
+      </c>
+      <c r="BJ50" t="s">
+        <v>90</v>
+      </c>
+      <c r="BK50">
+        <v>17</v>
+      </c>
+      <c r="BL50">
+        <v>16</v>
+      </c>
+      <c r="BM50">
+        <v>7</v>
+      </c>
+      <c r="BN50">
+        <v>8</v>
+      </c>
+      <c r="BO50">
+        <v>5</v>
+      </c>
+      <c r="BP50">
+        <v>3</v>
+      </c>
+      <c r="BQ50">
+        <v>21</v>
+      </c>
+      <c r="BR50">
+        <v>49</v>
+      </c>
+      <c r="BS50">
+        <v>6</v>
+      </c>
+      <c r="BT50">
+        <v>6</v>
+      </c>
+      <c r="BU50" t="s">
+        <v>90</v>
+      </c>
+      <c r="BV50" t="s">
+        <v>90</v>
+      </c>
+      <c r="BW50">
+        <v>48</v>
+      </c>
+      <c r="BX50">
+        <v>44</v>
+      </c>
+      <c r="BY50">
+        <v>29</v>
+      </c>
+      <c r="BZ50">
+        <v>28</v>
+      </c>
+      <c r="CA50">
+        <v>19</v>
+      </c>
+      <c r="CB50">
+        <v>16</v>
+      </c>
+      <c r="CC50">
+        <v>7</v>
+      </c>
+      <c r="CD50">
+        <v>5</v>
+      </c>
+      <c r="CE50" t="s">
+        <v>90</v>
+      </c>
+      <c r="CF50" t="s">
+        <v>90</v>
+      </c>
+      <c r="CG50">
+        <v>2</v>
+      </c>
+      <c r="CH50">
+        <v>1</v>
+      </c>
+      <c r="CI50">
+        <v>0</v>
+      </c>
+      <c r="CJ50">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="2:88" ht="25.5">
+      <c r="B51" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="C51" t="s">
+        <v>97</v>
+      </c>
+      <c r="D51" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="E51">
+        <v>1</v>
+      </c>
+      <c r="F51">
+        <v>0</v>
+      </c>
+      <c r="G51">
+        <v>62</v>
+      </c>
+      <c r="H51">
+        <f t="shared" si="0"/>
+        <v>38</v>
+      </c>
+      <c r="I51">
+        <v>1.37</v>
+      </c>
+      <c r="J51">
+        <v>0.46</v>
+      </c>
+      <c r="K51">
+        <v>16</v>
+      </c>
+      <c r="L51">
+        <v>8</v>
+      </c>
+      <c r="M51">
+        <v>6</v>
+      </c>
+      <c r="N51">
+        <v>1</v>
+      </c>
+      <c r="O51">
+        <v>2</v>
+      </c>
+      <c r="P51">
+        <v>0</v>
+      </c>
+      <c r="Q51">
+        <v>2</v>
+      </c>
+      <c r="R51">
+        <v>0</v>
+      </c>
+      <c r="S51">
+        <v>447</v>
+      </c>
+      <c r="T51">
+        <v>240</v>
+      </c>
+      <c r="U51">
+        <v>12</v>
+      </c>
+      <c r="V51">
+        <v>15</v>
+      </c>
+      <c r="W51">
+        <v>6</v>
+      </c>
+      <c r="X51">
+        <v>3</v>
+      </c>
+      <c r="Y51" t="s">
+        <v>90</v>
+      </c>
+      <c r="Z51" t="s">
+        <v>90</v>
+      </c>
+      <c r="AA51">
+        <v>6</v>
+      </c>
+      <c r="AB51">
+        <v>5</v>
+      </c>
+      <c r="AC51">
+        <v>4</v>
+      </c>
+      <c r="AD51">
+        <v>2</v>
+      </c>
+      <c r="AE51">
+        <v>1</v>
+      </c>
+      <c r="AF51">
+        <v>0</v>
+      </c>
+      <c r="AG51">
+        <v>9</v>
+      </c>
+      <c r="AH51">
+        <v>3</v>
+      </c>
+      <c r="AI51">
+        <v>7</v>
+      </c>
+      <c r="AJ51">
+        <v>5</v>
+      </c>
+      <c r="AK51">
+        <v>0.24</v>
+      </c>
+      <c r="AL51">
+        <v>0.24</v>
+      </c>
+      <c r="AM51">
+        <v>1.1299999999999999</v>
+      </c>
+      <c r="AN51">
+        <v>0.23</v>
+      </c>
+      <c r="AO51">
+        <v>1.37</v>
+      </c>
+      <c r="AP51">
+        <v>0.46</v>
+      </c>
+      <c r="AQ51">
+        <v>1</v>
+      </c>
+      <c r="AR51">
+        <v>0.65</v>
+      </c>
+      <c r="AS51">
+        <v>532</v>
+      </c>
+      <c r="AT51">
+        <v>333</v>
+      </c>
+      <c r="AU51">
+        <v>224</v>
+      </c>
+      <c r="AV51">
+        <v>157</v>
+      </c>
+      <c r="AW51">
+        <v>223</v>
+      </c>
+      <c r="AX51">
+        <v>83</v>
+      </c>
+      <c r="AY51">
+        <v>41</v>
+      </c>
+      <c r="AZ51">
+        <v>18</v>
+      </c>
+      <c r="BA51">
+        <v>9</v>
+      </c>
+      <c r="BB51">
+        <v>2</v>
+      </c>
+      <c r="BC51">
+        <v>20</v>
+      </c>
+      <c r="BD51">
+        <v>15</v>
+      </c>
+      <c r="BE51">
+        <v>36</v>
+      </c>
+      <c r="BF51">
+        <v>13</v>
+      </c>
+      <c r="BG51">
+        <v>2</v>
+      </c>
+      <c r="BH51">
+        <v>0</v>
+      </c>
+      <c r="BI51" t="s">
+        <v>90</v>
+      </c>
+      <c r="BJ51" t="s">
+        <v>90</v>
+      </c>
+      <c r="BK51">
+        <v>12</v>
+      </c>
+      <c r="BL51">
+        <v>22</v>
+      </c>
+      <c r="BM51">
+        <v>13</v>
+      </c>
+      <c r="BN51">
+        <v>12</v>
+      </c>
+      <c r="BO51">
+        <v>2</v>
+      </c>
+      <c r="BP51">
+        <v>4</v>
+      </c>
+      <c r="BQ51">
+        <v>23</v>
+      </c>
+      <c r="BR51">
+        <v>48</v>
+      </c>
+      <c r="BS51">
+        <v>1</v>
+      </c>
+      <c r="BT51">
+        <v>5</v>
+      </c>
+      <c r="BU51" t="s">
+        <v>90</v>
+      </c>
+      <c r="BV51" t="s">
+        <v>90</v>
+      </c>
+      <c r="BW51">
+        <v>55</v>
+      </c>
+      <c r="BX51">
+        <v>61</v>
+      </c>
+      <c r="BY51">
+        <v>29</v>
+      </c>
+      <c r="BZ51">
+        <v>43</v>
+      </c>
+      <c r="CA51">
+        <v>26</v>
+      </c>
+      <c r="CB51">
+        <v>18</v>
+      </c>
+      <c r="CC51">
+        <v>3</v>
+      </c>
+      <c r="CD51">
+        <v>10</v>
+      </c>
+      <c r="CE51" t="s">
+        <v>90</v>
+      </c>
+      <c r="CF51" t="s">
+        <v>90</v>
+      </c>
+      <c r="CG51">
+        <v>1</v>
+      </c>
+      <c r="CH51">
+        <v>2</v>
+      </c>
+      <c r="CI51">
+        <v>0</v>
+      </c>
+      <c r="CJ51">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="2:88" ht="25.5">
+      <c r="B52" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="C52" t="s">
+        <v>98</v>
+      </c>
+      <c r="D52" t="s">
+        <v>92</v>
+      </c>
+      <c r="E52">
+        <v>4</v>
+      </c>
+      <c r="F52">
+        <v>0</v>
+      </c>
+      <c r="G52">
+        <v>55</v>
+      </c>
+      <c r="H52">
+        <f t="shared" si="0"/>
+        <v>45</v>
+      </c>
+      <c r="I52">
+        <v>2.87</v>
+      </c>
+      <c r="J52">
+        <v>0.8</v>
+      </c>
+      <c r="K52">
+        <v>13</v>
+      </c>
+      <c r="L52">
+        <v>5</v>
+      </c>
+      <c r="M52">
+        <v>6</v>
+      </c>
+      <c r="N52">
+        <v>1</v>
+      </c>
+      <c r="O52">
+        <v>4</v>
+      </c>
+      <c r="P52">
+        <v>1</v>
+      </c>
+      <c r="Q52">
+        <v>1</v>
+      </c>
+      <c r="R52">
+        <v>1</v>
+      </c>
+      <c r="S52">
+        <v>403</v>
+      </c>
+      <c r="T52">
+        <v>319</v>
+      </c>
+      <c r="U52">
+        <v>10</v>
+      </c>
+      <c r="V52">
+        <v>18</v>
+      </c>
+      <c r="W52">
+        <v>4</v>
+      </c>
+      <c r="X52">
+        <v>6</v>
+      </c>
+      <c r="Y52" t="s">
+        <v>90</v>
+      </c>
+      <c r="Z52" t="s">
+        <v>90</v>
+      </c>
+      <c r="AA52">
+        <v>6</v>
+      </c>
+      <c r="AB52">
+        <v>4</v>
+      </c>
+      <c r="AC52">
+        <v>1</v>
+      </c>
+      <c r="AD52">
+        <v>0</v>
+      </c>
+      <c r="AE52">
+        <v>0</v>
+      </c>
+      <c r="AF52">
+        <v>0</v>
+      </c>
+      <c r="AG52">
+        <v>10</v>
+      </c>
+      <c r="AH52">
+        <v>3</v>
+      </c>
+      <c r="AI52">
+        <v>3</v>
+      </c>
+      <c r="AJ52">
+        <v>2</v>
+      </c>
+      <c r="AK52">
+        <v>2.12</v>
+      </c>
+      <c r="AL52">
+        <v>0.77</v>
+      </c>
+      <c r="AM52">
+        <v>0.75</v>
+      </c>
+      <c r="AN52">
+        <v>0.02</v>
+      </c>
+      <c r="AO52">
+        <v>2.87</v>
+      </c>
+      <c r="AP52">
+        <v>0.8</v>
+      </c>
+      <c r="AQ52">
+        <v>2.57</v>
+      </c>
+      <c r="AR52">
+        <v>0.03</v>
+      </c>
+      <c r="AS52">
+        <v>488</v>
+      </c>
+      <c r="AT52">
+        <v>394</v>
+      </c>
+      <c r="AU52">
+        <v>238</v>
+      </c>
+      <c r="AV52">
+        <v>223</v>
+      </c>
+      <c r="AW52">
+        <v>165</v>
+      </c>
+      <c r="AX52">
+        <v>96</v>
+      </c>
+      <c r="AY52">
+        <v>21</v>
+      </c>
+      <c r="AZ52">
+        <v>17</v>
+      </c>
+      <c r="BA52">
+        <v>1</v>
+      </c>
+      <c r="BB52">
+        <v>1</v>
+      </c>
+      <c r="BC52">
+        <v>16</v>
+      </c>
+      <c r="BD52">
+        <v>30</v>
+      </c>
+      <c r="BE52">
+        <v>22</v>
+      </c>
+      <c r="BF52">
+        <v>13</v>
+      </c>
+      <c r="BG52">
+        <v>0</v>
+      </c>
+      <c r="BH52">
+        <v>1</v>
+      </c>
+      <c r="BI52" t="s">
+        <v>90</v>
+      </c>
+      <c r="BJ52" t="s">
+        <v>90</v>
+      </c>
+      <c r="BK52">
+        <v>28</v>
+      </c>
+      <c r="BL52">
+        <v>18</v>
+      </c>
+      <c r="BM52">
+        <v>9</v>
+      </c>
+      <c r="BN52">
+        <v>18</v>
+      </c>
+      <c r="BO52">
+        <v>0</v>
+      </c>
+      <c r="BP52">
+        <v>1</v>
+      </c>
+      <c r="BQ52">
+        <v>16</v>
+      </c>
+      <c r="BR52">
+        <v>18</v>
+      </c>
+      <c r="BS52">
+        <v>1</v>
+      </c>
+      <c r="BT52">
+        <v>2</v>
+      </c>
+      <c r="BU52" t="s">
+        <v>90</v>
+      </c>
+      <c r="BV52" t="s">
+        <v>90</v>
+      </c>
+      <c r="BW52">
+        <v>66</v>
+      </c>
+      <c r="BX52">
+        <v>51</v>
+      </c>
+      <c r="BY52">
+        <v>55</v>
+      </c>
+      <c r="BZ52">
+        <v>40</v>
+      </c>
+      <c r="CA52">
+        <v>11</v>
+      </c>
+      <c r="CB52">
+        <v>11</v>
+      </c>
+      <c r="CC52">
+        <v>12</v>
+      </c>
+      <c r="CD52">
+        <v>12</v>
+      </c>
+      <c r="CE52" t="s">
+        <v>90</v>
+      </c>
+      <c r="CF52" t="s">
+        <v>90</v>
+      </c>
+      <c r="CG52">
+        <v>1</v>
+      </c>
+      <c r="CH52">
+        <v>1</v>
+      </c>
+      <c r="CI52">
+        <v>0</v>
+      </c>
+      <c r="CJ52">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="2:88" ht="25.5">
+      <c r="B53" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="D53" t="s">
+        <v>101</v>
+      </c>
+      <c r="E53">
+        <v>1</v>
+      </c>
+      <c r="F53">
+        <v>0</v>
+      </c>
+      <c r="G53">
+        <v>59</v>
+      </c>
+      <c r="H53">
+        <f t="shared" si="0"/>
+        <v>41</v>
+      </c>
+      <c r="I53">
+        <v>1.48</v>
+      </c>
+      <c r="J53">
+        <v>0.85</v>
+      </c>
+      <c r="K53">
+        <v>18</v>
+      </c>
+      <c r="L53">
+        <v>8</v>
+      </c>
+      <c r="M53">
+        <v>5</v>
+      </c>
+      <c r="N53">
+        <v>3</v>
+      </c>
+      <c r="O53">
+        <v>2</v>
+      </c>
+      <c r="P53">
+        <v>1</v>
+      </c>
+      <c r="Q53">
+        <v>2</v>
+      </c>
+      <c r="R53">
+        <v>1</v>
+      </c>
+      <c r="S53">
+        <v>384</v>
+      </c>
+      <c r="T53">
+        <v>270</v>
+      </c>
+      <c r="U53">
+        <v>7</v>
+      </c>
+      <c r="V53">
+        <v>12</v>
+      </c>
+      <c r="W53">
+        <v>13</v>
+      </c>
+      <c r="X53">
+        <v>1</v>
+      </c>
+      <c r="Y53" t="s">
+        <v>90</v>
+      </c>
+      <c r="Z53" t="s">
+        <v>90</v>
+      </c>
+      <c r="AA53">
+        <v>10</v>
+      </c>
+      <c r="AB53">
+        <v>4</v>
+      </c>
+      <c r="AC53">
+        <v>3</v>
+      </c>
+      <c r="AD53">
+        <v>1</v>
+      </c>
+      <c r="AE53">
+        <v>1</v>
+      </c>
+      <c r="AF53">
+        <v>0</v>
+      </c>
+      <c r="AG53">
+        <v>13</v>
+      </c>
+      <c r="AH53">
+        <v>4</v>
+      </c>
+      <c r="AI53">
+        <v>5</v>
+      </c>
+      <c r="AJ53">
+        <v>4</v>
+      </c>
+      <c r="AK53">
+        <v>0.66</v>
+      </c>
+      <c r="AL53">
+        <v>0.85</v>
+      </c>
+      <c r="AM53">
+        <v>0.83</v>
+      </c>
+      <c r="AN53">
+        <v>0</v>
+      </c>
+      <c r="AO53">
+        <v>1.48</v>
+      </c>
+      <c r="AP53">
+        <v>0.85</v>
+      </c>
+      <c r="AQ53">
+        <v>0.79</v>
+      </c>
+      <c r="AR53">
+        <v>0.7</v>
+      </c>
+      <c r="AS53">
+        <v>479</v>
+      </c>
+      <c r="AT53">
+        <v>357</v>
+      </c>
+      <c r="AU53">
+        <v>174</v>
+      </c>
+      <c r="AV53">
+        <v>157</v>
+      </c>
+      <c r="AW53">
+        <v>210</v>
+      </c>
+      <c r="AX53">
+        <v>113</v>
+      </c>
+      <c r="AY53">
+        <v>26</v>
+      </c>
+      <c r="AZ53">
+        <v>24</v>
+      </c>
+      <c r="BA53">
+        <v>6</v>
+      </c>
+      <c r="BB53">
+        <v>1</v>
+      </c>
+      <c r="BC53">
+        <v>37</v>
+      </c>
+      <c r="BD53">
+        <v>25</v>
+      </c>
+      <c r="BE53">
+        <v>36</v>
+      </c>
+      <c r="BF53">
+        <v>14</v>
+      </c>
+      <c r="BG53">
+        <v>1</v>
+      </c>
+      <c r="BH53">
+        <v>4</v>
+      </c>
+      <c r="BI53" t="s">
+        <v>90</v>
+      </c>
+      <c r="BJ53" t="s">
+        <v>90</v>
+      </c>
+      <c r="BK53">
+        <v>16</v>
+      </c>
+      <c r="BL53">
+        <v>16</v>
+      </c>
+      <c r="BM53">
+        <v>10</v>
+      </c>
+      <c r="BN53">
+        <v>11</v>
+      </c>
+      <c r="BO53">
+        <v>1</v>
+      </c>
+      <c r="BP53">
+        <v>2</v>
+      </c>
+      <c r="BQ53">
+        <v>27</v>
+      </c>
+      <c r="BR53">
+        <v>51</v>
+      </c>
+      <c r="BS53">
+        <v>3</v>
+      </c>
+      <c r="BT53">
+        <v>4</v>
+      </c>
+      <c r="BU53" t="s">
+        <v>90</v>
+      </c>
+      <c r="BV53" t="s">
+        <v>90</v>
+      </c>
+      <c r="BW53">
+        <v>51</v>
+      </c>
+      <c r="BX53">
+        <v>49</v>
+      </c>
+      <c r="BY53">
+        <v>33</v>
+      </c>
+      <c r="BZ53">
+        <v>32</v>
+      </c>
+      <c r="CA53">
+        <v>18</v>
+      </c>
+      <c r="CB53">
+        <v>17</v>
+      </c>
+      <c r="CC53">
+        <v>7</v>
+      </c>
+      <c r="CD53">
+        <v>9</v>
+      </c>
+      <c r="CE53" t="s">
+        <v>90</v>
+      </c>
+      <c r="CF53" t="s">
+        <v>90</v>
+      </c>
+      <c r="CG53">
+        <v>0</v>
+      </c>
+      <c r="CH53">
+        <v>2</v>
+      </c>
+      <c r="CI53">
+        <v>0</v>
+      </c>
+      <c r="CJ53">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Oct 31, 2026, 12:53 PM
</commit_message>
<xml_diff>
--- a/Bundesliga 26-27.xlsx
+++ b/Bundesliga 26-27.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kuba\Desktop\analityczka\26-27\Ekstraklasa 26-27\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{750824C8-E38B-4868-B529-6B406F92FDA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6E31CD27-8D71-49E4-90D2-302142366D49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{723BE2C8-720D-41E0-A496-B3B96A8488E1}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="659" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="681" uniqueCount="136">
   <si>
     <t>date</t>
   </si>
@@ -441,6 +441,12 @@
   </si>
   <si>
     <t>Sat 24 October, 18:30</t>
+  </si>
+  <si>
+    <t>Sun 25 October, 15:30</t>
+  </si>
+  <si>
+    <t>Sun 25 October, 17:30</t>
   </si>
 </sst>
 </file>
@@ -866,7 +872,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9ED51FE2-0441-4690-9385-28E7CF18BF79}">
-  <dimension ref="B1:CJ53"/>
+  <dimension ref="B1:CJ55"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="17.7109375" customWidth="1"/>
@@ -1187,7 +1193,7 @@
         <v>59</v>
       </c>
       <c r="H2">
-        <f t="shared" ref="H2:H53" si="0">100-G2</f>
+        <f t="shared" ref="H2:H55" si="0">100-G2</f>
         <v>41</v>
       </c>
       <c r="I2">
@@ -14892,6 +14898,534 @@
         <v>0</v>
       </c>
       <c r="CJ53">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="2:88" ht="25.5">
+      <c r="B54" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="C54" t="s">
+        <v>95</v>
+      </c>
+      <c r="D54" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="E54">
+        <v>0</v>
+      </c>
+      <c r="F54">
+        <v>0</v>
+      </c>
+      <c r="G54">
+        <v>42</v>
+      </c>
+      <c r="H54">
+        <f t="shared" si="0"/>
+        <v>58</v>
+      </c>
+      <c r="I54">
+        <v>3.46</v>
+      </c>
+      <c r="J54">
+        <v>0.56999999999999995</v>
+      </c>
+      <c r="K54">
+        <v>20</v>
+      </c>
+      <c r="L54">
+        <v>9</v>
+      </c>
+      <c r="M54">
+        <v>6</v>
+      </c>
+      <c r="N54">
+        <v>1</v>
+      </c>
+      <c r="O54">
+        <v>4</v>
+      </c>
+      <c r="P54">
+        <v>1</v>
+      </c>
+      <c r="Q54">
+        <v>1</v>
+      </c>
+      <c r="R54">
+        <v>1</v>
+      </c>
+      <c r="S54">
+        <v>279</v>
+      </c>
+      <c r="T54">
+        <v>432</v>
+      </c>
+      <c r="U54">
+        <v>14</v>
+      </c>
+      <c r="V54">
+        <v>6</v>
+      </c>
+      <c r="W54">
+        <v>5</v>
+      </c>
+      <c r="X54">
+        <v>3</v>
+      </c>
+      <c r="Y54" t="s">
+        <v>90</v>
+      </c>
+      <c r="Z54" t="s">
+        <v>90</v>
+      </c>
+      <c r="AA54">
+        <v>10</v>
+      </c>
+      <c r="AB54">
+        <v>6</v>
+      </c>
+      <c r="AC54">
+        <v>4</v>
+      </c>
+      <c r="AD54">
+        <v>2</v>
+      </c>
+      <c r="AE54">
+        <v>2</v>
+      </c>
+      <c r="AF54">
+        <v>0</v>
+      </c>
+      <c r="AG54">
+        <v>15</v>
+      </c>
+      <c r="AH54">
+        <v>6</v>
+      </c>
+      <c r="AI54">
+        <v>5</v>
+      </c>
+      <c r="AJ54">
+        <v>3</v>
+      </c>
+      <c r="AK54">
+        <v>2.34</v>
+      </c>
+      <c r="AL54">
+        <v>0.46</v>
+      </c>
+      <c r="AM54">
+        <v>0.33</v>
+      </c>
+      <c r="AN54">
+        <v>0.11</v>
+      </c>
+      <c r="AO54">
+        <v>2.67</v>
+      </c>
+      <c r="AP54">
+        <v>0.56999999999999995</v>
+      </c>
+      <c r="AQ54">
+        <v>2.2400000000000002</v>
+      </c>
+      <c r="AR54">
+        <v>0.22</v>
+      </c>
+      <c r="AS54">
+        <v>359</v>
+      </c>
+      <c r="AT54">
+        <v>509</v>
+      </c>
+      <c r="AU54">
+        <v>139</v>
+      </c>
+      <c r="AV54">
+        <v>203</v>
+      </c>
+      <c r="AW54">
+        <v>140</v>
+      </c>
+      <c r="AX54">
+        <v>229</v>
+      </c>
+      <c r="AY54">
+        <v>18</v>
+      </c>
+      <c r="AZ54">
+        <v>23</v>
+      </c>
+      <c r="BA54">
+        <v>5</v>
+      </c>
+      <c r="BB54">
+        <v>1</v>
+      </c>
+      <c r="BC54">
+        <v>18</v>
+      </c>
+      <c r="BD54">
+        <v>22</v>
+      </c>
+      <c r="BE54">
+        <v>28</v>
+      </c>
+      <c r="BF54">
+        <v>20</v>
+      </c>
+      <c r="BG54">
+        <v>1</v>
+      </c>
+      <c r="BH54">
+        <v>0</v>
+      </c>
+      <c r="BI54" t="s">
+        <v>90</v>
+      </c>
+      <c r="BJ54" t="s">
+        <v>90</v>
+      </c>
+      <c r="BK54">
+        <v>15</v>
+      </c>
+      <c r="BL54">
+        <v>15</v>
+      </c>
+      <c r="BM54">
+        <v>16</v>
+      </c>
+      <c r="BN54">
+        <v>11</v>
+      </c>
+      <c r="BO54">
+        <v>2</v>
+      </c>
+      <c r="BP54">
+        <v>4</v>
+      </c>
+      <c r="BQ54">
+        <v>32</v>
+      </c>
+      <c r="BR54">
+        <v>18</v>
+      </c>
+      <c r="BS54">
+        <v>1</v>
+      </c>
+      <c r="BT54">
+        <v>3</v>
+      </c>
+      <c r="BU54" t="s">
+        <v>90</v>
+      </c>
+      <c r="BV54" t="s">
+        <v>90</v>
+      </c>
+      <c r="BW54">
+        <v>42</v>
+      </c>
+      <c r="BX54">
+        <v>43</v>
+      </c>
+      <c r="BY54">
+        <v>28</v>
+      </c>
+      <c r="BZ54">
+        <v>35</v>
+      </c>
+      <c r="CA54">
+        <v>14</v>
+      </c>
+      <c r="CB54">
+        <v>8</v>
+      </c>
+      <c r="CC54">
+        <v>7</v>
+      </c>
+      <c r="CD54">
+        <v>7</v>
+      </c>
+      <c r="CE54" t="s">
+        <v>90</v>
+      </c>
+      <c r="CF54" t="s">
+        <v>90</v>
+      </c>
+      <c r="CG54">
+        <v>2</v>
+      </c>
+      <c r="CH54">
+        <v>4</v>
+      </c>
+      <c r="CI54">
+        <v>1</v>
+      </c>
+      <c r="CJ54">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="2:88" ht="25.5">
+      <c r="B55" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="C55" t="s">
+        <v>106</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E55">
+        <v>1</v>
+      </c>
+      <c r="F55">
+        <v>3</v>
+      </c>
+      <c r="G55">
+        <v>44</v>
+      </c>
+      <c r="H55">
+        <f t="shared" si="0"/>
+        <v>56</v>
+      </c>
+      <c r="I55">
+        <v>1.01</v>
+      </c>
+      <c r="J55">
+        <v>2.91</v>
+      </c>
+      <c r="K55">
+        <v>16</v>
+      </c>
+      <c r="L55">
+        <v>17</v>
+      </c>
+      <c r="M55">
+        <v>4</v>
+      </c>
+      <c r="N55">
+        <v>9</v>
+      </c>
+      <c r="O55">
+        <v>0</v>
+      </c>
+      <c r="P55">
+        <v>6</v>
+      </c>
+      <c r="Q55">
+        <v>0</v>
+      </c>
+      <c r="R55">
+        <v>3</v>
+      </c>
+      <c r="S55">
+        <v>333</v>
+      </c>
+      <c r="T55">
+        <v>442</v>
+      </c>
+      <c r="U55">
+        <v>9</v>
+      </c>
+      <c r="V55">
+        <v>11</v>
+      </c>
+      <c r="W55">
+        <v>5</v>
+      </c>
+      <c r="X55">
+        <v>6</v>
+      </c>
+      <c r="Y55" t="s">
+        <v>90</v>
+      </c>
+      <c r="Z55" t="s">
+        <v>90</v>
+      </c>
+      <c r="AA55">
+        <v>5</v>
+      </c>
+      <c r="AB55">
+        <v>7</v>
+      </c>
+      <c r="AC55">
+        <v>7</v>
+      </c>
+      <c r="AD55">
+        <v>1</v>
+      </c>
+      <c r="AE55">
+        <v>0</v>
+      </c>
+      <c r="AF55">
+        <v>0</v>
+      </c>
+      <c r="AG55">
+        <v>8</v>
+      </c>
+      <c r="AH55">
+        <v>12</v>
+      </c>
+      <c r="AI55">
+        <v>8</v>
+      </c>
+      <c r="AJ55">
+        <v>5</v>
+      </c>
+      <c r="AK55">
+        <v>0.59</v>
+      </c>
+      <c r="AL55">
+        <v>2.41</v>
+      </c>
+      <c r="AM55">
+        <v>0.42</v>
+      </c>
+      <c r="AN55">
+        <v>0.5</v>
+      </c>
+      <c r="AO55">
+        <v>1.01</v>
+      </c>
+      <c r="AP55">
+        <v>2.91</v>
+      </c>
+      <c r="AQ55">
+        <v>1.05</v>
+      </c>
+      <c r="AR55">
+        <v>3.22</v>
+      </c>
+      <c r="AS55">
+        <v>407</v>
+      </c>
+      <c r="AT55">
+        <v>523</v>
+      </c>
+      <c r="AU55">
+        <v>206</v>
+      </c>
+      <c r="AV55">
+        <v>242</v>
+      </c>
+      <c r="AW55">
+        <v>127</v>
+      </c>
+      <c r="AX55">
+        <v>200</v>
+      </c>
+      <c r="AY55">
+        <v>14</v>
+      </c>
+      <c r="AZ55">
+        <v>25</v>
+      </c>
+      <c r="BA55">
+        <v>5</v>
+      </c>
+      <c r="BB55">
+        <v>2</v>
+      </c>
+      <c r="BC55">
+        <v>9</v>
+      </c>
+      <c r="BD55">
+        <v>17</v>
+      </c>
+      <c r="BE55">
+        <v>25</v>
+      </c>
+      <c r="BF55">
+        <v>22</v>
+      </c>
+      <c r="BG55">
+        <v>1</v>
+      </c>
+      <c r="BH55">
+        <v>1</v>
+      </c>
+      <c r="BI55" t="s">
+        <v>90</v>
+      </c>
+      <c r="BJ55" t="s">
+        <v>90</v>
+      </c>
+      <c r="BK55">
+        <v>19</v>
+      </c>
+      <c r="BL55">
+        <v>19</v>
+      </c>
+      <c r="BM55">
+        <v>8</v>
+      </c>
+      <c r="BN55">
+        <v>4</v>
+      </c>
+      <c r="BO55">
+        <v>1</v>
+      </c>
+      <c r="BP55">
+        <v>6</v>
+      </c>
+      <c r="BQ55">
+        <v>16</v>
+      </c>
+      <c r="BR55">
+        <v>23</v>
+      </c>
+      <c r="BS55">
+        <v>6</v>
+      </c>
+      <c r="BT55">
+        <v>4</v>
+      </c>
+      <c r="BU55" t="s">
+        <v>90</v>
+      </c>
+      <c r="BV55" t="s">
+        <v>90</v>
+      </c>
+      <c r="BW55">
+        <v>50</v>
+      </c>
+      <c r="BX55">
+        <v>47</v>
+      </c>
+      <c r="BY55">
+        <v>37</v>
+      </c>
+      <c r="BZ55">
+        <v>38</v>
+      </c>
+      <c r="CA55">
+        <v>13</v>
+      </c>
+      <c r="CB55">
+        <v>9</v>
+      </c>
+      <c r="CC55">
+        <v>8</v>
+      </c>
+      <c r="CD55">
+        <v>10</v>
+      </c>
+      <c r="CE55" t="s">
+        <v>90</v>
+      </c>
+      <c r="CF55" t="s">
+        <v>90</v>
+      </c>
+      <c r="CG55">
+        <v>3</v>
+      </c>
+      <c r="CH55">
+        <v>1</v>
+      </c>
+      <c r="CI55">
+        <v>0</v>
+      </c>
+      <c r="CJ55">
         <v>0</v>
       </c>
     </row>

</xml_diff>